<commit_message>
i have change the codes of the transfer the and corrected the grand total tally
</commit_message>
<xml_diff>
--- a/backend/db/transfer/overall_data.xlsx
+++ b/backend/db/transfer/overall_data.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1417">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1435">
   <si>
     <t>admission</t>
   </si>
@@ -3511,6 +3511,9 @@
     <t>LKG</t>
   </si>
   <si>
+    <t>09/02/2025</t>
+  </si>
+  <si>
     <t>MOHAMMED RIFAZ M</t>
   </si>
   <si>
@@ -4268,6 +4271,57 @@
   </si>
   <si>
     <t>22/08/2024</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>amount</t>
+  </si>
+  <si>
+    <t>total</t>
+  </si>
+  <si>
+    <t>mode</t>
+  </si>
+  <si>
+    <t>new admission application</t>
+  </si>
+  <si>
+    <t>04/02/2025</t>
+  </si>
+  <si>
+    <t>cash</t>
+  </si>
+  <si>
+    <t>id card</t>
+  </si>
+  <si>
+    <t>belt,id card</t>
+  </si>
+  <si>
+    <t>50,100</t>
+  </si>
+  <si>
+    <t>05/02/2025</t>
+  </si>
+  <si>
+    <t>term iii</t>
+  </si>
+  <si>
+    <t>cheque_online</t>
+  </si>
+  <si>
+    <t>bonafide certificate</t>
+  </si>
+  <si>
+    <t>belt</t>
+  </si>
+  <si>
+    <t>06/02/2025</t>
+  </si>
+  <si>
+    <t>term ii</t>
   </si>
 </sst>
 </file>
@@ -22088,7 +22142,7 @@
         <v>26985</v>
       </c>
       <c r="N372">
-        <v>9000</v>
+        <v>26985</v>
       </c>
       <c r="O372">
         <v>0</v>
@@ -22840,7 +22894,7 @@
         <v>24685</v>
       </c>
       <c r="N388">
-        <v>0</v>
+        <v>24685</v>
       </c>
       <c r="O388">
         <v>0</v>
@@ -22981,7 +23035,7 @@
         <v>24685</v>
       </c>
       <c r="N391">
-        <v>0</v>
+        <v>24685</v>
       </c>
       <c r="O391">
         <v>0</v>
@@ -25989,7 +26043,7 @@
         <v>22690</v>
       </c>
       <c r="N455">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O455">
         <v>0</v>
@@ -27164,7 +27218,7 @@
         <v>22690</v>
       </c>
       <c r="N480">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O480">
         <v>0</v>
@@ -27211,7 +27265,7 @@
         <v>22690</v>
       </c>
       <c r="N481">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O481">
         <v>0</v>
@@ -27446,7 +27500,7 @@
         <v>22690</v>
       </c>
       <c r="N486">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O486">
         <v>0</v>
@@ -27493,7 +27547,7 @@
         <v>22690</v>
       </c>
       <c r="N487">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O487">
         <v>0</v>
@@ -28903,7 +28957,7 @@
         <v>22690</v>
       </c>
       <c r="N517">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O517">
         <v>0</v>
@@ -28950,7 +29004,7 @@
         <v>22690</v>
       </c>
       <c r="N518">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O518">
         <v>0</v>
@@ -28997,7 +29051,7 @@
         <v>22690</v>
       </c>
       <c r="N519">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O519">
         <v>0</v>
@@ -29044,7 +29098,7 @@
         <v>22690</v>
       </c>
       <c r="N520">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O520">
         <v>0</v>
@@ -29091,7 +29145,7 @@
         <v>22690</v>
       </c>
       <c r="N521">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O521">
         <v>0</v>
@@ -29138,7 +29192,7 @@
         <v>22690</v>
       </c>
       <c r="N522">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O522">
         <v>0</v>
@@ -29185,7 +29239,7 @@
         <v>22690</v>
       </c>
       <c r="N523">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O523">
         <v>0</v>
@@ -29232,7 +29286,7 @@
         <v>22690</v>
       </c>
       <c r="N524">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O524">
         <v>0</v>
@@ -34120,7 +34174,7 @@
         <v>22690</v>
       </c>
       <c r="N628">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O628">
         <v>0</v>
@@ -34167,7 +34221,7 @@
         <v>22690</v>
       </c>
       <c r="N629">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O629">
         <v>0</v>
@@ -34214,7 +34268,7 @@
         <v>22690</v>
       </c>
       <c r="N630">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O630">
         <v>0</v>
@@ -34261,7 +34315,7 @@
         <v>22690</v>
       </c>
       <c r="N631">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O631">
         <v>0</v>
@@ -34308,7 +34362,7 @@
         <v>22690</v>
       </c>
       <c r="N632">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O632">
         <v>0</v>
@@ -34355,7 +34409,7 @@
         <v>22690</v>
       </c>
       <c r="N633">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O633">
         <v>0</v>
@@ -34402,7 +34456,7 @@
         <v>22690</v>
       </c>
       <c r="N634">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O634">
         <v>0</v>
@@ -34449,7 +34503,7 @@
         <v>22690</v>
       </c>
       <c r="N635">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O635">
         <v>0</v>
@@ -34543,7 +34597,7 @@
         <v>22690</v>
       </c>
       <c r="N637">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O637">
         <v>0</v>
@@ -35154,7 +35208,7 @@
         <v>22690</v>
       </c>
       <c r="N650">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O650">
         <v>0</v>
@@ -35201,7 +35255,7 @@
         <v>22690</v>
       </c>
       <c r="N651">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O651">
         <v>0</v>
@@ -35248,7 +35302,7 @@
         <v>22690</v>
       </c>
       <c r="N652">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O652">
         <v>0</v>
@@ -35295,7 +35349,7 @@
         <v>22690</v>
       </c>
       <c r="N653">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O653">
         <v>0</v>
@@ -35342,7 +35396,7 @@
         <v>22690</v>
       </c>
       <c r="N654">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O654">
         <v>0</v>
@@ -35389,7 +35443,7 @@
         <v>22690</v>
       </c>
       <c r="N655">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O655">
         <v>0</v>
@@ -35436,7 +35490,7 @@
         <v>22690</v>
       </c>
       <c r="N656">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O656">
         <v>0</v>
@@ -35483,7 +35537,7 @@
         <v>22690</v>
       </c>
       <c r="N657">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O657">
         <v>0</v>
@@ -35530,7 +35584,7 @@
         <v>22690</v>
       </c>
       <c r="N658">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O658">
         <v>0</v>
@@ -35577,7 +35631,7 @@
         <v>22690</v>
       </c>
       <c r="N659">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O659">
         <v>0</v>
@@ -35624,7 +35678,7 @@
         <v>22690</v>
       </c>
       <c r="N660">
-        <v>0</v>
+        <v>22690</v>
       </c>
       <c r="O660">
         <v>0</v>
@@ -44695,7 +44749,7 @@
         <v>20330</v>
       </c>
       <c r="N853">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O853">
         <v>0</v>
@@ -44742,7 +44796,7 @@
         <v>20330</v>
       </c>
       <c r="N854">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O854">
         <v>0</v>
@@ -44789,7 +44843,7 @@
         <v>20330</v>
       </c>
       <c r="N855">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O855">
         <v>0</v>
@@ -44836,7 +44890,7 @@
         <v>20330</v>
       </c>
       <c r="N856">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O856">
         <v>0</v>
@@ -44883,7 +44937,7 @@
         <v>20330</v>
       </c>
       <c r="N857">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O857">
         <v>0</v>
@@ -44930,7 +44984,7 @@
         <v>20330</v>
       </c>
       <c r="N858">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O858">
         <v>0</v>
@@ -44977,7 +45031,7 @@
         <v>20330</v>
       </c>
       <c r="N859">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O859">
         <v>0</v>
@@ -45024,7 +45078,7 @@
         <v>20330</v>
       </c>
       <c r="N860">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O860">
         <v>0</v>
@@ -45071,7 +45125,7 @@
         <v>20330</v>
       </c>
       <c r="N861">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O861">
         <v>0</v>
@@ -45118,7 +45172,7 @@
         <v>20330</v>
       </c>
       <c r="N862">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O862">
         <v>0</v>
@@ -45165,7 +45219,7 @@
         <v>20330</v>
       </c>
       <c r="N863">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O863">
         <v>0</v>
@@ -45212,7 +45266,7 @@
         <v>20330</v>
       </c>
       <c r="N864">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O864">
         <v>0</v>
@@ -45259,7 +45313,7 @@
         <v>20330</v>
       </c>
       <c r="N865">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O865">
         <v>0</v>
@@ -45306,7 +45360,7 @@
         <v>20330</v>
       </c>
       <c r="N866">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O866">
         <v>0</v>
@@ -54594,7 +54648,7 @@
         <v>0</v>
       </c>
       <c r="H1064" t="s">
-        <v>44</v>
+        <v>1164</v>
       </c>
       <c r="I1064" t="s">
         <v>462</v>
@@ -54603,19 +54657,19 @@
         <v>20330</v>
       </c>
       <c r="K1064">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="L1064">
         <v>0</v>
       </c>
       <c r="M1064">
+        <v>23330</v>
+      </c>
+      <c r="N1064">
         <v>20330</v>
       </c>
-      <c r="N1064">
-        <v>0</v>
-      </c>
       <c r="O1064">
-        <v>0</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="1065" spans="1:15">
@@ -54623,7 +54677,7 @@
         <v>8840</v>
       </c>
       <c r="B1065" t="s">
-        <v>1164</v>
+        <v>1165</v>
       </c>
       <c r="C1065" t="s">
         <v>1163</v>
@@ -54659,7 +54713,7 @@
         <v>20330</v>
       </c>
       <c r="N1065">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O1065">
         <v>0</v>
@@ -54670,7 +54724,7 @@
         <v>8841</v>
       </c>
       <c r="B1066" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="C1066" t="s">
         <v>1163</v>
@@ -54706,7 +54760,7 @@
         <v>20330</v>
       </c>
       <c r="N1066">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O1066">
         <v>0</v>
@@ -54717,7 +54771,7 @@
         <v>8842</v>
       </c>
       <c r="B1067" t="s">
-        <v>1166</v>
+        <v>1167</v>
       </c>
       <c r="C1067" t="s">
         <v>1163</v>
@@ -54753,7 +54807,7 @@
         <v>20330</v>
       </c>
       <c r="N1067">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O1067">
         <v>0</v>
@@ -54764,7 +54818,7 @@
         <v>8843</v>
       </c>
       <c r="B1068" t="s">
-        <v>1167</v>
+        <v>1168</v>
       </c>
       <c r="C1068" t="s">
         <v>1163</v>
@@ -54800,7 +54854,7 @@
         <v>20330</v>
       </c>
       <c r="N1068">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O1068">
         <v>0</v>
@@ -54811,7 +54865,7 @@
         <v>8844</v>
       </c>
       <c r="B1069" t="s">
-        <v>1168</v>
+        <v>1169</v>
       </c>
       <c r="C1069" t="s">
         <v>1163</v>
@@ -54847,7 +54901,7 @@
         <v>20330</v>
       </c>
       <c r="N1069">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O1069">
         <v>0</v>
@@ -54894,7 +54948,7 @@
         <v>20330</v>
       </c>
       <c r="N1070">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O1070">
         <v>0</v>
@@ -54905,7 +54959,7 @@
         <v>8846</v>
       </c>
       <c r="B1071" t="s">
-        <v>1169</v>
+        <v>1170</v>
       </c>
       <c r="C1071" t="s">
         <v>1163</v>
@@ -54941,7 +54995,7 @@
         <v>20330</v>
       </c>
       <c r="N1071">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O1071">
         <v>0</v>
@@ -54952,7 +55006,7 @@
         <v>8847</v>
       </c>
       <c r="B1072" t="s">
-        <v>1170</v>
+        <v>1171</v>
       </c>
       <c r="C1072" t="s">
         <v>1163</v>
@@ -54988,7 +55042,7 @@
         <v>20330</v>
       </c>
       <c r="N1072">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O1072">
         <v>0</v>
@@ -54999,7 +55053,7 @@
         <v>8848</v>
       </c>
       <c r="B1073" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="C1073" t="s">
         <v>1163</v>
@@ -55035,7 +55089,7 @@
         <v>20330</v>
       </c>
       <c r="N1073">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O1073">
         <v>0</v>
@@ -55046,7 +55100,7 @@
         <v>8849</v>
       </c>
       <c r="B1074" t="s">
-        <v>1172</v>
+        <v>1173</v>
       </c>
       <c r="C1074" t="s">
         <v>1163</v>
@@ -55082,7 +55136,7 @@
         <v>20330</v>
       </c>
       <c r="N1074">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O1074">
         <v>0</v>
@@ -55093,7 +55147,7 @@
         <v>8850</v>
       </c>
       <c r="B1075" t="s">
-        <v>1173</v>
+        <v>1174</v>
       </c>
       <c r="C1075" t="s">
         <v>1163</v>
@@ -55129,7 +55183,7 @@
         <v>20330</v>
       </c>
       <c r="N1075">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O1075">
         <v>0</v>
@@ -55140,7 +55194,7 @@
         <v>8851</v>
       </c>
       <c r="B1076" t="s">
-        <v>1174</v>
+        <v>1175</v>
       </c>
       <c r="C1076" t="s">
         <v>1163</v>
@@ -55176,7 +55230,7 @@
         <v>20330</v>
       </c>
       <c r="N1076">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O1076">
         <v>0</v>
@@ -55187,7 +55241,7 @@
         <v>8852</v>
       </c>
       <c r="B1077" t="s">
-        <v>1175</v>
+        <v>1176</v>
       </c>
       <c r="C1077" t="s">
         <v>1163</v>
@@ -55223,7 +55277,7 @@
         <v>20330</v>
       </c>
       <c r="N1077">
-        <v>0</v>
+        <v>20330</v>
       </c>
       <c r="O1077">
         <v>0</v>
@@ -55234,7 +55288,7 @@
         <v>8854</v>
       </c>
       <c r="B1078" t="s">
-        <v>1176</v>
+        <v>1177</v>
       </c>
       <c r="C1078" t="s">
         <v>1163</v>
@@ -55252,7 +55306,7 @@
         <v>0</v>
       </c>
       <c r="H1078" t="s">
-        <v>1177</v>
+        <v>1178</v>
       </c>
       <c r="I1078" t="s">
         <v>19</v>
@@ -55281,7 +55335,7 @@
         <v>8855</v>
       </c>
       <c r="B1079" t="s">
-        <v>1178</v>
+        <v>1179</v>
       </c>
       <c r="C1079" t="s">
         <v>1163</v>
@@ -55299,7 +55353,7 @@
         <v>0</v>
       </c>
       <c r="H1079" t="s">
-        <v>1177</v>
+        <v>1178</v>
       </c>
       <c r="I1079" t="s">
         <v>19</v>
@@ -55328,7 +55382,7 @@
         <v>8857</v>
       </c>
       <c r="B1080" t="s">
-        <v>1179</v>
+        <v>1180</v>
       </c>
       <c r="C1080" t="s">
         <v>1163</v>
@@ -55346,7 +55400,7 @@
         <v>0</v>
       </c>
       <c r="H1080" t="s">
-        <v>1180</v>
+        <v>1181</v>
       </c>
       <c r="I1080" t="s">
         <v>19</v>
@@ -55375,7 +55429,7 @@
         <v>8858</v>
       </c>
       <c r="B1081" t="s">
-        <v>1181</v>
+        <v>1182</v>
       </c>
       <c r="C1081" t="s">
         <v>1163</v>
@@ -55393,7 +55447,7 @@
         <v>0</v>
       </c>
       <c r="H1081" t="s">
-        <v>1180</v>
+        <v>1181</v>
       </c>
       <c r="I1081" t="s">
         <v>19</v>
@@ -55422,7 +55476,7 @@
         <v>8859</v>
       </c>
       <c r="B1082" t="s">
-        <v>1182</v>
+        <v>1183</v>
       </c>
       <c r="C1082" t="s">
         <v>1163</v>
@@ -55440,7 +55494,7 @@
         <v>0</v>
       </c>
       <c r="H1082" t="s">
-        <v>1183</v>
+        <v>1184</v>
       </c>
       <c r="I1082" t="s">
         <v>19</v>
@@ -55469,7 +55523,7 @@
         <v>8860</v>
       </c>
       <c r="B1083" t="s">
-        <v>1184</v>
+        <v>1185</v>
       </c>
       <c r="C1083" t="s">
         <v>1163</v>
@@ -55487,7 +55541,7 @@
         <v>0</v>
       </c>
       <c r="H1083" t="s">
-        <v>1185</v>
+        <v>1186</v>
       </c>
       <c r="I1083" t="s">
         <v>19</v>
@@ -55516,7 +55570,7 @@
         <v>8861</v>
       </c>
       <c r="B1084" t="s">
-        <v>1186</v>
+        <v>1187</v>
       </c>
       <c r="C1084" t="s">
         <v>1163</v>
@@ -55534,7 +55588,7 @@
         <v>0</v>
       </c>
       <c r="H1084" t="s">
-        <v>1187</v>
+        <v>1188</v>
       </c>
       <c r="I1084" t="s">
         <v>19</v>
@@ -55563,7 +55617,7 @@
         <v>8862</v>
       </c>
       <c r="B1085" t="s">
-        <v>1188</v>
+        <v>1189</v>
       </c>
       <c r="C1085" t="s">
         <v>1163</v>
@@ -55610,7 +55664,7 @@
         <v>8863</v>
       </c>
       <c r="B1086" t="s">
-        <v>1189</v>
+        <v>1190</v>
       </c>
       <c r="C1086" t="s">
         <v>1163</v>
@@ -55628,7 +55682,7 @@
         <v>0</v>
       </c>
       <c r="H1086" t="s">
-        <v>1185</v>
+        <v>1186</v>
       </c>
       <c r="I1086" t="s">
         <v>19</v>
@@ -55657,7 +55711,7 @@
         <v>8864</v>
       </c>
       <c r="B1087" t="s">
-        <v>1190</v>
+        <v>1191</v>
       </c>
       <c r="C1087" t="s">
         <v>1163</v>
@@ -55675,7 +55729,7 @@
         <v>0</v>
       </c>
       <c r="H1087" t="s">
-        <v>1191</v>
+        <v>1192</v>
       </c>
       <c r="I1087" t="s">
         <v>19</v>
@@ -55704,7 +55758,7 @@
         <v>8865</v>
       </c>
       <c r="B1088" t="s">
-        <v>1192</v>
+        <v>1193</v>
       </c>
       <c r="C1088" t="s">
         <v>1163</v>
@@ -55722,7 +55776,7 @@
         <v>0</v>
       </c>
       <c r="H1088" t="s">
-        <v>1193</v>
+        <v>1194</v>
       </c>
       <c r="I1088" t="s">
         <v>19</v>
@@ -55751,7 +55805,7 @@
         <v>8866</v>
       </c>
       <c r="B1089" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="C1089" t="s">
         <v>1163</v>
@@ -55798,7 +55852,7 @@
         <v>8867</v>
       </c>
       <c r="B1090" t="s">
-        <v>1195</v>
+        <v>1196</v>
       </c>
       <c r="C1090" t="s">
         <v>1163</v>
@@ -55845,7 +55899,7 @@
         <v>8868</v>
       </c>
       <c r="B1091" t="s">
-        <v>1196</v>
+        <v>1197</v>
       </c>
       <c r="C1091" t="s">
         <v>1163</v>
@@ -55892,7 +55946,7 @@
         <v>8869</v>
       </c>
       <c r="B1092" t="s">
-        <v>1197</v>
+        <v>1198</v>
       </c>
       <c r="C1092" t="s">
         <v>1163</v>
@@ -55939,7 +55993,7 @@
         <v>8870</v>
       </c>
       <c r="B1093" t="s">
-        <v>1198</v>
+        <v>1199</v>
       </c>
       <c r="C1093" t="s">
         <v>1163</v>
@@ -55986,7 +56040,7 @@
         <v>8871</v>
       </c>
       <c r="B1094" t="s">
-        <v>1199</v>
+        <v>1200</v>
       </c>
       <c r="C1094" t="s">
         <v>1163</v>
@@ -56033,7 +56087,7 @@
         <v>8872</v>
       </c>
       <c r="B1095" t="s">
-        <v>1200</v>
+        <v>1201</v>
       </c>
       <c r="C1095" t="s">
         <v>1163</v>
@@ -56080,7 +56134,7 @@
         <v>8873</v>
       </c>
       <c r="B1096" t="s">
-        <v>1201</v>
+        <v>1202</v>
       </c>
       <c r="C1096" t="s">
         <v>1163</v>
@@ -56127,7 +56181,7 @@
         <v>8874</v>
       </c>
       <c r="B1097" t="s">
-        <v>1202</v>
+        <v>1203</v>
       </c>
       <c r="C1097" t="s">
         <v>1163</v>
@@ -56174,7 +56228,7 @@
         <v>8875</v>
       </c>
       <c r="B1098" t="s">
-        <v>1203</v>
+        <v>1204</v>
       </c>
       <c r="C1098" t="s">
         <v>1163</v>
@@ -56221,7 +56275,7 @@
         <v>8876</v>
       </c>
       <c r="B1099" t="s">
-        <v>1204</v>
+        <v>1205</v>
       </c>
       <c r="C1099" t="s">
         <v>1163</v>
@@ -56268,7 +56322,7 @@
         <v>8877</v>
       </c>
       <c r="B1100" t="s">
-        <v>1205</v>
+        <v>1206</v>
       </c>
       <c r="C1100" t="s">
         <v>1163</v>
@@ -56315,7 +56369,7 @@
         <v>8878</v>
       </c>
       <c r="B1101" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="C1101" t="s">
         <v>1163</v>
@@ -56362,7 +56416,7 @@
         <v>8879</v>
       </c>
       <c r="B1102" t="s">
-        <v>1207</v>
+        <v>1208</v>
       </c>
       <c r="C1102" t="s">
         <v>1163</v>
@@ -56409,7 +56463,7 @@
         <v>8880</v>
       </c>
       <c r="B1103" t="s">
-        <v>1208</v>
+        <v>1209</v>
       </c>
       <c r="C1103" t="s">
         <v>1163</v>
@@ -56456,7 +56510,7 @@
         <v>8881</v>
       </c>
       <c r="B1104" t="s">
-        <v>1209</v>
+        <v>1210</v>
       </c>
       <c r="C1104" t="s">
         <v>1163</v>
@@ -56503,7 +56557,7 @@
         <v>8882</v>
       </c>
       <c r="B1105" t="s">
-        <v>1210</v>
+        <v>1211</v>
       </c>
       <c r="C1105" t="s">
         <v>1163</v>
@@ -56550,7 +56604,7 @@
         <v>8883</v>
       </c>
       <c r="B1106" t="s">
-        <v>1211</v>
+        <v>1212</v>
       </c>
       <c r="C1106" t="s">
         <v>1163</v>
@@ -56597,7 +56651,7 @@
         <v>8884</v>
       </c>
       <c r="B1107" t="s">
-        <v>1212</v>
+        <v>1213</v>
       </c>
       <c r="C1107" t="s">
         <v>1163</v>
@@ -56644,7 +56698,7 @@
         <v>8885</v>
       </c>
       <c r="B1108" t="s">
-        <v>1213</v>
+        <v>1214</v>
       </c>
       <c r="C1108" t="s">
         <v>1163</v>
@@ -56691,7 +56745,7 @@
         <v>8886</v>
       </c>
       <c r="B1109" t="s">
-        <v>1214</v>
+        <v>1215</v>
       </c>
       <c r="C1109" t="s">
         <v>1163</v>
@@ -56738,7 +56792,7 @@
         <v>8887</v>
       </c>
       <c r="B1110" t="s">
-        <v>1215</v>
+        <v>1216</v>
       </c>
       <c r="C1110" t="s">
         <v>1163</v>
@@ -56785,7 +56839,7 @@
         <v>8888</v>
       </c>
       <c r="B1111" t="s">
-        <v>1216</v>
+        <v>1217</v>
       </c>
       <c r="C1111" t="s">
         <v>952</v>
@@ -56803,7 +56857,7 @@
         <v>0</v>
       </c>
       <c r="H1111" t="s">
-        <v>1177</v>
+        <v>1178</v>
       </c>
       <c r="I1111" t="s">
         <v>19</v>
@@ -56832,7 +56886,7 @@
         <v>8889</v>
       </c>
       <c r="B1112" t="s">
-        <v>1217</v>
+        <v>1218</v>
       </c>
       <c r="C1112" t="s">
         <v>952</v>
@@ -56850,7 +56904,7 @@
         <v>0</v>
       </c>
       <c r="H1112" t="s">
-        <v>1218</v>
+        <v>1219</v>
       </c>
       <c r="I1112" t="s">
         <v>19</v>
@@ -56879,7 +56933,7 @@
         <v>8890</v>
       </c>
       <c r="B1113" t="s">
-        <v>1219</v>
+        <v>1220</v>
       </c>
       <c r="C1113" t="s">
         <v>952</v>
@@ -56897,7 +56951,7 @@
         <v>0</v>
       </c>
       <c r="H1113" t="s">
-        <v>1180</v>
+        <v>1181</v>
       </c>
       <c r="I1113" t="s">
         <v>19</v>
@@ -56926,7 +56980,7 @@
         <v>8891</v>
       </c>
       <c r="B1114" t="s">
-        <v>1220</v>
+        <v>1221</v>
       </c>
       <c r="C1114" t="s">
         <v>952</v>
@@ -56973,7 +57027,7 @@
         <v>8892</v>
       </c>
       <c r="B1115" t="s">
-        <v>1221</v>
+        <v>1222</v>
       </c>
       <c r="C1115" t="s">
         <v>952</v>
@@ -56991,7 +57045,7 @@
         <v>0</v>
       </c>
       <c r="H1115" t="s">
-        <v>1222</v>
+        <v>1223</v>
       </c>
       <c r="I1115" t="s">
         <v>19</v>
@@ -57020,7 +57074,7 @@
         <v>8893</v>
       </c>
       <c r="B1116" t="s">
-        <v>1223</v>
+        <v>1224</v>
       </c>
       <c r="C1116" t="s">
         <v>952</v>
@@ -57067,7 +57121,7 @@
         <v>8894</v>
       </c>
       <c r="B1117" t="s">
-        <v>1224</v>
+        <v>1225</v>
       </c>
       <c r="C1117" t="s">
         <v>952</v>
@@ -57114,7 +57168,7 @@
         <v>8895</v>
       </c>
       <c r="B1118" t="s">
-        <v>1225</v>
+        <v>1226</v>
       </c>
       <c r="C1118" t="s">
         <v>952</v>
@@ -57161,7 +57215,7 @@
         <v>8896</v>
       </c>
       <c r="B1119" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C1119" t="s">
         <v>952</v>
@@ -57208,7 +57262,7 @@
         <v>8897</v>
       </c>
       <c r="B1120" t="s">
-        <v>1227</v>
+        <v>1228</v>
       </c>
       <c r="C1120" t="s">
         <v>952</v>
@@ -57255,7 +57309,7 @@
         <v>8898</v>
       </c>
       <c r="B1121" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
       <c r="C1121" t="s">
         <v>952</v>
@@ -57302,7 +57356,7 @@
         <v>8899</v>
       </c>
       <c r="B1122" t="s">
-        <v>1229</v>
+        <v>1230</v>
       </c>
       <c r="C1122" t="s">
         <v>952</v>
@@ -57349,7 +57403,7 @@
         <v>8900</v>
       </c>
       <c r="B1123" t="s">
-        <v>1230</v>
+        <v>1231</v>
       </c>
       <c r="C1123" t="s">
         <v>749</v>
@@ -57367,7 +57421,7 @@
         <v>0</v>
       </c>
       <c r="H1123" t="s">
-        <v>1231</v>
+        <v>1232</v>
       </c>
       <c r="I1123" t="s">
         <v>19</v>
@@ -57396,7 +57450,7 @@
         <v>8901</v>
       </c>
       <c r="B1124" t="s">
-        <v>1232</v>
+        <v>1233</v>
       </c>
       <c r="C1124" t="s">
         <v>749</v>
@@ -57414,7 +57468,7 @@
         <v>0</v>
       </c>
       <c r="H1124" t="s">
-        <v>1233</v>
+        <v>1234</v>
       </c>
       <c r="I1124" t="s">
         <v>19</v>
@@ -57443,7 +57497,7 @@
         <v>8902</v>
       </c>
       <c r="B1125" t="s">
-        <v>1234</v>
+        <v>1235</v>
       </c>
       <c r="C1125" t="s">
         <v>749</v>
@@ -57461,7 +57515,7 @@
         <v>0</v>
       </c>
       <c r="H1125" t="s">
-        <v>1235</v>
+        <v>1236</v>
       </c>
       <c r="I1125" t="s">
         <v>19</v>
@@ -57490,7 +57544,7 @@
         <v>8903</v>
       </c>
       <c r="B1126" t="s">
-        <v>1236</v>
+        <v>1237</v>
       </c>
       <c r="C1126" t="s">
         <v>749</v>
@@ -57537,7 +57591,7 @@
         <v>8904</v>
       </c>
       <c r="B1127" t="s">
-        <v>1237</v>
+        <v>1238</v>
       </c>
       <c r="C1127" t="s">
         <v>749</v>
@@ -57584,7 +57638,7 @@
         <v>8905</v>
       </c>
       <c r="B1128" t="s">
-        <v>1238</v>
+        <v>1239</v>
       </c>
       <c r="C1128" t="s">
         <v>749</v>
@@ -57631,7 +57685,7 @@
         <v>8906</v>
       </c>
       <c r="B1129" t="s">
-        <v>1239</v>
+        <v>1240</v>
       </c>
       <c r="C1129" t="s">
         <v>749</v>
@@ -57678,7 +57732,7 @@
         <v>8907</v>
       </c>
       <c r="B1130" t="s">
-        <v>1240</v>
+        <v>1241</v>
       </c>
       <c r="C1130" t="s">
         <v>749</v>
@@ -57725,7 +57779,7 @@
         <v>8908</v>
       </c>
       <c r="B1131" t="s">
-        <v>1241</v>
+        <v>1242</v>
       </c>
       <c r="C1131" t="s">
         <v>749</v>
@@ -57772,7 +57826,7 @@
         <v>8909</v>
       </c>
       <c r="B1132" t="s">
-        <v>1242</v>
+        <v>1243</v>
       </c>
       <c r="C1132" t="s">
         <v>749</v>
@@ -57819,7 +57873,7 @@
         <v>8910</v>
       </c>
       <c r="B1133" t="s">
-        <v>1243</v>
+        <v>1244</v>
       </c>
       <c r="C1133" t="s">
         <v>749</v>
@@ -57866,7 +57920,7 @@
         <v>8911</v>
       </c>
       <c r="B1134" t="s">
-        <v>1244</v>
+        <v>1245</v>
       </c>
       <c r="C1134" t="s">
         <v>749</v>
@@ -57913,7 +57967,7 @@
         <v>8912</v>
       </c>
       <c r="B1135" t="s">
-        <v>1245</v>
+        <v>1246</v>
       </c>
       <c r="C1135" t="s">
         <v>749</v>
@@ -57960,7 +58014,7 @@
         <v>8913</v>
       </c>
       <c r="B1136" t="s">
-        <v>1246</v>
+        <v>1247</v>
       </c>
       <c r="C1136" t="s">
         <v>749</v>
@@ -58007,7 +58061,7 @@
         <v>8914</v>
       </c>
       <c r="B1137" t="s">
-        <v>1247</v>
+        <v>1248</v>
       </c>
       <c r="C1137" t="s">
         <v>749</v>
@@ -58054,7 +58108,7 @@
         <v>8915</v>
       </c>
       <c r="B1138" t="s">
-        <v>1248</v>
+        <v>1249</v>
       </c>
       <c r="C1138" t="s">
         <v>656</v>
@@ -58072,7 +58126,7 @@
         <v>0</v>
       </c>
       <c r="H1138" t="s">
-        <v>1185</v>
+        <v>1186</v>
       </c>
       <c r="I1138" t="s">
         <v>19</v>
@@ -58101,7 +58155,7 @@
         <v>8916</v>
       </c>
       <c r="B1139" t="s">
-        <v>1249</v>
+        <v>1250</v>
       </c>
       <c r="C1139" t="s">
         <v>656</v>
@@ -58119,7 +58173,7 @@
         <v>0</v>
       </c>
       <c r="H1139" t="s">
-        <v>1231</v>
+        <v>1232</v>
       </c>
       <c r="I1139" t="s">
         <v>19</v>
@@ -58148,7 +58202,7 @@
         <v>8917</v>
       </c>
       <c r="B1140" t="s">
-        <v>1250</v>
+        <v>1251</v>
       </c>
       <c r="C1140" t="s">
         <v>656</v>
@@ -58195,7 +58249,7 @@
         <v>8918</v>
       </c>
       <c r="B1141" t="s">
-        <v>1251</v>
+        <v>1252</v>
       </c>
       <c r="C1141" t="s">
         <v>656</v>
@@ -58289,7 +58343,7 @@
         <v>8920</v>
       </c>
       <c r="B1143" t="s">
-        <v>1252</v>
+        <v>1253</v>
       </c>
       <c r="C1143" t="s">
         <v>656</v>
@@ -58336,7 +58390,7 @@
         <v>8921</v>
       </c>
       <c r="B1144" t="s">
-        <v>1253</v>
+        <v>1254</v>
       </c>
       <c r="C1144" t="s">
         <v>656</v>
@@ -58383,7 +58437,7 @@
         <v>8922</v>
       </c>
       <c r="B1145" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="C1145" t="s">
         <v>656</v>
@@ -58430,7 +58484,7 @@
         <v>8923</v>
       </c>
       <c r="B1146" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="C1146" t="s">
         <v>656</v>
@@ -58477,7 +58531,7 @@
         <v>8924</v>
       </c>
       <c r="B1147" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
       <c r="C1147" t="s">
         <v>656</v>
@@ -58524,7 +58578,7 @@
         <v>8925</v>
       </c>
       <c r="B1148" t="s">
-        <v>1257</v>
+        <v>1258</v>
       </c>
       <c r="C1148" t="s">
         <v>656</v>
@@ -58571,7 +58625,7 @@
         <v>8926</v>
       </c>
       <c r="B1149" t="s">
-        <v>1258</v>
+        <v>1259</v>
       </c>
       <c r="C1149" t="s">
         <v>656</v>
@@ -58618,7 +58672,7 @@
         <v>8927</v>
       </c>
       <c r="B1150" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="C1150" t="s">
         <v>656</v>
@@ -58665,7 +58719,7 @@
         <v>8928</v>
       </c>
       <c r="B1151" t="s">
-        <v>1260</v>
+        <v>1261</v>
       </c>
       <c r="C1151" t="s">
         <v>537</v>
@@ -58683,7 +58737,7 @@
         <v>7690</v>
       </c>
       <c r="H1151" t="s">
-        <v>1261</v>
+        <v>1262</v>
       </c>
       <c r="I1151" t="s">
         <v>19</v>
@@ -58712,7 +58766,7 @@
         <v>8929</v>
       </c>
       <c r="B1152" t="s">
-        <v>1262</v>
+        <v>1263</v>
       </c>
       <c r="C1152" t="s">
         <v>537</v>
@@ -58730,7 +58784,7 @@
         <v>0</v>
       </c>
       <c r="H1152" t="s">
-        <v>1218</v>
+        <v>1219</v>
       </c>
       <c r="I1152" t="s">
         <v>19</v>
@@ -58759,7 +58813,7 @@
         <v>8930</v>
       </c>
       <c r="B1153" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="C1153" t="s">
         <v>537</v>
@@ -58777,7 +58831,7 @@
         <v>0</v>
       </c>
       <c r="H1153" t="s">
-        <v>1235</v>
+        <v>1236</v>
       </c>
       <c r="I1153" t="s">
         <v>19</v>
@@ -58806,7 +58860,7 @@
         <v>8931</v>
       </c>
       <c r="B1154" t="s">
-        <v>1264</v>
+        <v>1265</v>
       </c>
       <c r="C1154" t="s">
         <v>537</v>
@@ -58824,7 +58878,7 @@
         <v>0</v>
       </c>
       <c r="H1154" t="s">
-        <v>1222</v>
+        <v>1223</v>
       </c>
       <c r="I1154" t="s">
         <v>19</v>
@@ -58853,7 +58907,7 @@
         <v>8932</v>
       </c>
       <c r="B1155" t="s">
-        <v>1265</v>
+        <v>1266</v>
       </c>
       <c r="C1155" t="s">
         <v>537</v>
@@ -58900,7 +58954,7 @@
         <v>8933</v>
       </c>
       <c r="B1156" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="C1156" t="s">
         <v>537</v>
@@ -58947,7 +59001,7 @@
         <v>8934</v>
       </c>
       <c r="B1157" t="s">
-        <v>1267</v>
+        <v>1268</v>
       </c>
       <c r="C1157" t="s">
         <v>537</v>
@@ -58994,7 +59048,7 @@
         <v>8935</v>
       </c>
       <c r="B1158" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="C1158" t="s">
         <v>537</v>
@@ -59041,7 +59095,7 @@
         <v>8936</v>
       </c>
       <c r="B1159" t="s">
-        <v>1269</v>
+        <v>1270</v>
       </c>
       <c r="C1159" t="s">
         <v>537</v>
@@ -59088,7 +59142,7 @@
         <v>8937</v>
       </c>
       <c r="B1160" t="s">
-        <v>1270</v>
+        <v>1271</v>
       </c>
       <c r="C1160" t="s">
         <v>537</v>
@@ -59135,7 +59189,7 @@
         <v>8938</v>
       </c>
       <c r="B1161" t="s">
-        <v>1271</v>
+        <v>1272</v>
       </c>
       <c r="C1161" t="s">
         <v>537</v>
@@ -59182,7 +59236,7 @@
         <v>8939</v>
       </c>
       <c r="B1162" t="s">
-        <v>1272</v>
+        <v>1273</v>
       </c>
       <c r="C1162" t="s">
         <v>537</v>
@@ -59229,7 +59283,7 @@
         <v>8940</v>
       </c>
       <c r="B1163" t="s">
-        <v>1273</v>
+        <v>1274</v>
       </c>
       <c r="C1163" t="s">
         <v>537</v>
@@ -59276,7 +59330,7 @@
         <v>8941</v>
       </c>
       <c r="B1164" t="s">
-        <v>1274</v>
+        <v>1275</v>
       </c>
       <c r="C1164" t="s">
         <v>537</v>
@@ -59323,7 +59377,7 @@
         <v>8942</v>
       </c>
       <c r="B1165" t="s">
-        <v>1275</v>
+        <v>1276</v>
       </c>
       <c r="C1165" t="s">
         <v>550</v>
@@ -59370,7 +59424,7 @@
         <v>8943</v>
       </c>
       <c r="B1166" t="s">
-        <v>1276</v>
+        <v>1277</v>
       </c>
       <c r="C1166" t="s">
         <v>550</v>
@@ -59388,7 +59442,7 @@
         <v>0</v>
       </c>
       <c r="H1166" t="s">
-        <v>1277</v>
+        <v>1278</v>
       </c>
       <c r="I1166" t="s">
         <v>19</v>
@@ -59417,7 +59471,7 @@
         <v>8944</v>
       </c>
       <c r="B1167" t="s">
-        <v>1278</v>
+        <v>1279</v>
       </c>
       <c r="C1167" t="s">
         <v>550</v>
@@ -59464,7 +59518,7 @@
         <v>8945</v>
       </c>
       <c r="B1168" t="s">
-        <v>1279</v>
+        <v>1280</v>
       </c>
       <c r="C1168" t="s">
         <v>550</v>
@@ -59511,7 +59565,7 @@
         <v>8946</v>
       </c>
       <c r="B1169" t="s">
-        <v>1280</v>
+        <v>1281</v>
       </c>
       <c r="C1169" t="s">
         <v>550</v>
@@ -59558,7 +59612,7 @@
         <v>8947</v>
       </c>
       <c r="B1170" t="s">
-        <v>1281</v>
+        <v>1282</v>
       </c>
       <c r="C1170" t="s">
         <v>550</v>
@@ -59605,7 +59659,7 @@
         <v>8948</v>
       </c>
       <c r="B1171" t="s">
-        <v>1282</v>
+        <v>1283</v>
       </c>
       <c r="C1171" t="s">
         <v>550</v>
@@ -59652,7 +59706,7 @@
         <v>8949</v>
       </c>
       <c r="B1172" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
       <c r="C1172" t="s">
         <v>550</v>
@@ -59699,7 +59753,7 @@
         <v>8950</v>
       </c>
       <c r="B1173" t="s">
-        <v>1284</v>
+        <v>1285</v>
       </c>
       <c r="C1173" t="s">
         <v>550</v>
@@ -59746,7 +59800,7 @@
         <v>8951</v>
       </c>
       <c r="B1174" t="s">
-        <v>1285</v>
+        <v>1286</v>
       </c>
       <c r="C1174" t="s">
         <v>497</v>
@@ -59764,7 +59818,7 @@
         <v>0</v>
       </c>
       <c r="H1174" t="s">
-        <v>1180</v>
+        <v>1181</v>
       </c>
       <c r="I1174" t="s">
         <v>19</v>
@@ -59793,7 +59847,7 @@
         <v>8952</v>
       </c>
       <c r="B1175" t="s">
-        <v>1286</v>
+        <v>1287</v>
       </c>
       <c r="C1175" t="s">
         <v>497</v>
@@ -59840,7 +59894,7 @@
         <v>8953</v>
       </c>
       <c r="B1176" t="s">
-        <v>1287</v>
+        <v>1288</v>
       </c>
       <c r="C1176" t="s">
         <v>497</v>
@@ -59887,7 +59941,7 @@
         <v>8954</v>
       </c>
       <c r="B1177" t="s">
-        <v>1288</v>
+        <v>1289</v>
       </c>
       <c r="C1177" t="s">
         <v>497</v>
@@ -59934,7 +59988,7 @@
         <v>8955</v>
       </c>
       <c r="B1178" t="s">
-        <v>1289</v>
+        <v>1290</v>
       </c>
       <c r="C1178" t="s">
         <v>497</v>
@@ -59981,7 +60035,7 @@
         <v>8956</v>
       </c>
       <c r="B1179" t="s">
-        <v>1290</v>
+        <v>1291</v>
       </c>
       <c r="C1179" t="s">
         <v>497</v>
@@ -60028,7 +60082,7 @@
         <v>8957</v>
       </c>
       <c r="B1180" t="s">
-        <v>1291</v>
+        <v>1292</v>
       </c>
       <c r="C1180" t="s">
         <v>497</v>
@@ -60075,7 +60129,7 @@
         <v>8958</v>
       </c>
       <c r="B1181" t="s">
-        <v>1292</v>
+        <v>1293</v>
       </c>
       <c r="C1181" t="s">
         <v>497</v>
@@ -60122,7 +60176,7 @@
         <v>8959</v>
       </c>
       <c r="B1182" t="s">
-        <v>1293</v>
+        <v>1294</v>
       </c>
       <c r="C1182" t="s">
         <v>497</v>
@@ -60169,7 +60223,7 @@
         <v>8960</v>
       </c>
       <c r="B1183" t="s">
-        <v>1294</v>
+        <v>1295</v>
       </c>
       <c r="C1183" t="s">
         <v>497</v>
@@ -60216,7 +60270,7 @@
         <v>8961</v>
       </c>
       <c r="B1184" t="s">
-        <v>1295</v>
+        <v>1296</v>
       </c>
       <c r="C1184" t="s">
         <v>497</v>
@@ -60263,7 +60317,7 @@
         <v>8962</v>
       </c>
       <c r="B1185" t="s">
-        <v>1296</v>
+        <v>1297</v>
       </c>
       <c r="C1185" t="s">
         <v>497</v>
@@ -60310,7 +60364,7 @@
         <v>8963</v>
       </c>
       <c r="B1186" t="s">
-        <v>1297</v>
+        <v>1298</v>
       </c>
       <c r="C1186" t="s">
         <v>497</v>
@@ -60357,7 +60411,7 @@
         <v>8964</v>
       </c>
       <c r="B1187" t="s">
-        <v>1298</v>
+        <v>1299</v>
       </c>
       <c r="C1187" t="s">
         <v>497</v>
@@ -60404,7 +60458,7 @@
         <v>8965</v>
       </c>
       <c r="B1188" t="s">
-        <v>1299</v>
+        <v>1300</v>
       </c>
       <c r="C1188" t="s">
         <v>464</v>
@@ -60451,7 +60505,7 @@
         <v>8966</v>
       </c>
       <c r="B1189" t="s">
-        <v>1300</v>
+        <v>1301</v>
       </c>
       <c r="C1189" t="s">
         <v>464</v>
@@ -60469,7 +60523,7 @@
         <v>0</v>
       </c>
       <c r="H1189" t="s">
-        <v>1277</v>
+        <v>1278</v>
       </c>
       <c r="I1189" t="s">
         <v>19</v>
@@ -60498,7 +60552,7 @@
         <v>8967</v>
       </c>
       <c r="B1190" t="s">
-        <v>1301</v>
+        <v>1302</v>
       </c>
       <c r="C1190" t="s">
         <v>464</v>
@@ -60545,7 +60599,7 @@
         <v>8968</v>
       </c>
       <c r="B1191" t="s">
-        <v>1302</v>
+        <v>1303</v>
       </c>
       <c r="C1191" t="s">
         <v>464</v>
@@ -60592,7 +60646,7 @@
         <v>8969</v>
       </c>
       <c r="B1192" t="s">
-        <v>1303</v>
+        <v>1304</v>
       </c>
       <c r="C1192" t="s">
         <v>464</v>
@@ -60639,7 +60693,7 @@
         <v>8970</v>
       </c>
       <c r="B1193" t="s">
-        <v>1304</v>
+        <v>1305</v>
       </c>
       <c r="C1193" t="s">
         <v>464</v>
@@ -60686,7 +60740,7 @@
         <v>8971</v>
       </c>
       <c r="B1194" t="s">
-        <v>1305</v>
+        <v>1306</v>
       </c>
       <c r="C1194" t="s">
         <v>464</v>
@@ -60733,7 +60787,7 @@
         <v>8972</v>
       </c>
       <c r="B1195" t="s">
-        <v>1306</v>
+        <v>1307</v>
       </c>
       <c r="C1195" t="s">
         <v>464</v>
@@ -60780,7 +60834,7 @@
         <v>8973</v>
       </c>
       <c r="B1196" t="s">
-        <v>1307</v>
+        <v>1308</v>
       </c>
       <c r="C1196" t="s">
         <v>464</v>
@@ -60827,7 +60881,7 @@
         <v>8974</v>
       </c>
       <c r="B1197" t="s">
-        <v>1308</v>
+        <v>1309</v>
       </c>
       <c r="C1197" t="s">
         <v>464</v>
@@ -60874,7 +60928,7 @@
         <v>8975</v>
       </c>
       <c r="B1198" t="s">
-        <v>1309</v>
+        <v>1310</v>
       </c>
       <c r="C1198" t="s">
         <v>464</v>
@@ -60921,7 +60975,7 @@
         <v>8976</v>
       </c>
       <c r="B1199" t="s">
-        <v>1310</v>
+        <v>1311</v>
       </c>
       <c r="C1199" t="s">
         <v>464</v>
@@ -60968,7 +61022,7 @@
         <v>8977</v>
       </c>
       <c r="B1200" t="s">
-        <v>1311</v>
+        <v>1312</v>
       </c>
       <c r="C1200" t="s">
         <v>464</v>
@@ -61015,7 +61069,7 @@
         <v>8978</v>
       </c>
       <c r="B1201" t="s">
-        <v>1312</v>
+        <v>1313</v>
       </c>
       <c r="C1201" t="s">
         <v>464</v>
@@ -61062,7 +61116,7 @@
         <v>8979</v>
       </c>
       <c r="B1202" t="s">
-        <v>1313</v>
+        <v>1314</v>
       </c>
       <c r="C1202" t="s">
         <v>464</v>
@@ -61109,7 +61163,7 @@
         <v>8980</v>
       </c>
       <c r="B1203" t="s">
-        <v>1314</v>
+        <v>1315</v>
       </c>
       <c r="C1203" t="s">
         <v>464</v>
@@ -61156,7 +61210,7 @@
         <v>8981</v>
       </c>
       <c r="B1204" t="s">
-        <v>1315</v>
+        <v>1316</v>
       </c>
       <c r="C1204" t="s">
         <v>464</v>
@@ -61203,7 +61257,7 @@
         <v>8982</v>
       </c>
       <c r="B1205" t="s">
-        <v>1316</v>
+        <v>1317</v>
       </c>
       <c r="C1205" t="s">
         <v>464</v>
@@ -61250,7 +61304,7 @@
         <v>8983</v>
       </c>
       <c r="B1206" t="s">
-        <v>1317</v>
+        <v>1318</v>
       </c>
       <c r="C1206" t="s">
         <v>464</v>
@@ -61297,7 +61351,7 @@
         <v>8984</v>
       </c>
       <c r="B1207" t="s">
-        <v>1318</v>
+        <v>1319</v>
       </c>
       <c r="C1207" t="s">
         <v>464</v>
@@ -61344,7 +61398,7 @@
         <v>8985</v>
       </c>
       <c r="B1208" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
       <c r="C1208" t="s">
         <v>464</v>
@@ -61391,7 +61445,7 @@
         <v>8986</v>
       </c>
       <c r="B1209" t="s">
-        <v>1320</v>
+        <v>1321</v>
       </c>
       <c r="C1209" t="s">
         <v>464</v>
@@ -61438,7 +61492,7 @@
         <v>8987</v>
       </c>
       <c r="B1210" t="s">
-        <v>1321</v>
+        <v>1322</v>
       </c>
       <c r="C1210" t="s">
         <v>464</v>
@@ -61485,7 +61539,7 @@
         <v>8988</v>
       </c>
       <c r="B1211" t="s">
-        <v>1322</v>
+        <v>1323</v>
       </c>
       <c r="C1211" t="s">
         <v>464</v>
@@ -61532,7 +61586,7 @@
         <v>8989</v>
       </c>
       <c r="B1212" t="s">
-        <v>1323</v>
+        <v>1324</v>
       </c>
       <c r="C1212" t="s">
         <v>464</v>
@@ -61579,7 +61633,7 @@
         <v>8990</v>
       </c>
       <c r="B1213" t="s">
-        <v>1324</v>
+        <v>1325</v>
       </c>
       <c r="C1213" t="s">
         <v>464</v>
@@ -61626,7 +61680,7 @@
         <v>8991</v>
       </c>
       <c r="B1214" t="s">
-        <v>1325</v>
+        <v>1326</v>
       </c>
       <c r="C1214" t="s">
         <v>464</v>
@@ -61673,7 +61727,7 @@
         <v>8992</v>
       </c>
       <c r="B1215" t="s">
-        <v>1326</v>
+        <v>1327</v>
       </c>
       <c r="C1215" t="s">
         <v>464</v>
@@ -61720,7 +61774,7 @@
         <v>8993</v>
       </c>
       <c r="B1216" t="s">
-        <v>1327</v>
+        <v>1328</v>
       </c>
       <c r="C1216" t="s">
         <v>464</v>
@@ -61767,7 +61821,7 @@
         <v>8994</v>
       </c>
       <c r="B1217" t="s">
-        <v>1328</v>
+        <v>1329</v>
       </c>
       <c r="C1217" t="s">
         <v>464</v>
@@ -61814,7 +61868,7 @@
         <v>8995</v>
       </c>
       <c r="B1218" t="s">
-        <v>1329</v>
+        <v>1330</v>
       </c>
       <c r="C1218" t="s">
         <v>464</v>
@@ -61861,7 +61915,7 @@
         <v>8996</v>
       </c>
       <c r="B1219" t="s">
-        <v>1330</v>
+        <v>1331</v>
       </c>
       <c r="C1219" t="s">
         <v>464</v>
@@ -61908,7 +61962,7 @@
         <v>8997</v>
       </c>
       <c r="B1220" t="s">
-        <v>1331</v>
+        <v>1332</v>
       </c>
       <c r="C1220" t="s">
         <v>464</v>
@@ -61955,7 +62009,7 @@
         <v>8998</v>
       </c>
       <c r="B1221" t="s">
-        <v>1332</v>
+        <v>1333</v>
       </c>
       <c r="C1221" t="s">
         <v>464</v>
@@ -62002,7 +62056,7 @@
         <v>8999</v>
       </c>
       <c r="B1222" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="C1222" t="s">
         <v>464</v>
@@ -62049,7 +62103,7 @@
         <v>9000</v>
       </c>
       <c r="B1223" t="s">
-        <v>1334</v>
+        <v>1335</v>
       </c>
       <c r="C1223" t="s">
         <v>464</v>
@@ -62096,7 +62150,7 @@
         <v>9001</v>
       </c>
       <c r="B1224" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="C1224" t="s">
         <v>464</v>
@@ -62190,7 +62244,7 @@
         <v>9003</v>
       </c>
       <c r="B1226" t="s">
-        <v>1336</v>
+        <v>1337</v>
       </c>
       <c r="C1226" t="s">
         <v>427</v>
@@ -62208,7 +62262,7 @@
         <v>0</v>
       </c>
       <c r="H1226" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="I1226" t="s">
         <v>19</v>
@@ -62237,7 +62291,7 @@
         <v>9004</v>
       </c>
       <c r="B1227" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="C1227" t="s">
         <v>427</v>
@@ -62284,7 +62338,7 @@
         <v>9005</v>
       </c>
       <c r="B1228" t="s">
-        <v>1339</v>
+        <v>1340</v>
       </c>
       <c r="C1228" t="s">
         <v>427</v>
@@ -62331,7 +62385,7 @@
         <v>9006</v>
       </c>
       <c r="B1229" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="C1229" t="s">
         <v>427</v>
@@ -62378,7 +62432,7 @@
         <v>9007</v>
       </c>
       <c r="B1230" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="C1230" t="s">
         <v>427</v>
@@ -62425,7 +62479,7 @@
         <v>9008</v>
       </c>
       <c r="B1231" t="s">
-        <v>1342</v>
+        <v>1343</v>
       </c>
       <c r="C1231" t="s">
         <v>427</v>
@@ -62472,7 +62526,7 @@
         <v>9009</v>
       </c>
       <c r="B1232" t="s">
-        <v>1343</v>
+        <v>1344</v>
       </c>
       <c r="C1232" t="s">
         <v>427</v>
@@ -62519,7 +62573,7 @@
         <v>9010</v>
       </c>
       <c r="B1233" t="s">
-        <v>1344</v>
+        <v>1345</v>
       </c>
       <c r="C1233" t="s">
         <v>427</v>
@@ -62566,7 +62620,7 @@
         <v>9011</v>
       </c>
       <c r="B1234" t="s">
-        <v>1345</v>
+        <v>1346</v>
       </c>
       <c r="C1234" t="s">
         <v>427</v>
@@ -62613,7 +62667,7 @@
         <v>9012</v>
       </c>
       <c r="B1235" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="C1235" t="s">
         <v>427</v>
@@ -62660,7 +62714,7 @@
         <v>9013</v>
       </c>
       <c r="B1236" t="s">
-        <v>1347</v>
+        <v>1348</v>
       </c>
       <c r="C1236" t="s">
         <v>427</v>
@@ -62707,7 +62761,7 @@
         <v>9014</v>
       </c>
       <c r="B1237" t="s">
-        <v>1348</v>
+        <v>1349</v>
       </c>
       <c r="C1237" t="s">
         <v>427</v>
@@ -62754,7 +62808,7 @@
         <v>9015</v>
       </c>
       <c r="B1238" t="s">
-        <v>1349</v>
+        <v>1350</v>
       </c>
       <c r="C1238" t="s">
         <v>427</v>
@@ -62801,7 +62855,7 @@
         <v>9016</v>
       </c>
       <c r="B1239" t="s">
-        <v>1350</v>
+        <v>1351</v>
       </c>
       <c r="C1239" t="s">
         <v>427</v>
@@ -62848,7 +62902,7 @@
         <v>9017</v>
       </c>
       <c r="B1240" t="s">
-        <v>1351</v>
+        <v>1352</v>
       </c>
       <c r="C1240" t="s">
         <v>427</v>
@@ -62895,7 +62949,7 @@
         <v>9018</v>
       </c>
       <c r="B1241" t="s">
-        <v>1352</v>
+        <v>1353</v>
       </c>
       <c r="C1241" t="s">
         <v>427</v>
@@ -62942,7 +62996,7 @@
         <v>9019</v>
       </c>
       <c r="B1242" t="s">
-        <v>1353</v>
+        <v>1354</v>
       </c>
       <c r="C1242" t="s">
         <v>427</v>
@@ -62989,7 +63043,7 @@
         <v>9020</v>
       </c>
       <c r="B1243" t="s">
-        <v>1354</v>
+        <v>1355</v>
       </c>
       <c r="C1243" t="s">
         <v>427</v>
@@ -63036,7 +63090,7 @@
         <v>9021</v>
       </c>
       <c r="B1244" t="s">
-        <v>1355</v>
+        <v>1356</v>
       </c>
       <c r="C1244" t="s">
         <v>427</v>
@@ -63083,7 +63137,7 @@
         <v>9022</v>
       </c>
       <c r="B1245" t="s">
-        <v>1356</v>
+        <v>1357</v>
       </c>
       <c r="C1245" t="s">
         <v>427</v>
@@ -63130,7 +63184,7 @@
         <v>9023</v>
       </c>
       <c r="B1246" t="s">
-        <v>1357</v>
+        <v>1358</v>
       </c>
       <c r="C1246" t="s">
         <v>427</v>
@@ -63177,7 +63231,7 @@
         <v>9024</v>
       </c>
       <c r="B1247" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="C1247" t="s">
         <v>393</v>
@@ -63195,7 +63249,7 @@
         <v>0</v>
       </c>
       <c r="H1247" t="s">
-        <v>1222</v>
+        <v>1223</v>
       </c>
       <c r="I1247" t="s">
         <v>19</v>
@@ -63224,7 +63278,7 @@
         <v>9025</v>
       </c>
       <c r="B1248" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
       <c r="C1248" t="s">
         <v>393</v>
@@ -63242,7 +63296,7 @@
         <v>0</v>
       </c>
       <c r="H1248" t="s">
-        <v>1222</v>
+        <v>1223</v>
       </c>
       <c r="I1248" t="s">
         <v>19</v>
@@ -63271,7 +63325,7 @@
         <v>9026</v>
       </c>
       <c r="B1249" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
       <c r="C1249" t="s">
         <v>393</v>
@@ -63318,7 +63372,7 @@
         <v>9027</v>
       </c>
       <c r="B1250" t="s">
-        <v>1361</v>
+        <v>1362</v>
       </c>
       <c r="C1250" t="s">
         <v>393</v>
@@ -63365,7 +63419,7 @@
         <v>9028</v>
       </c>
       <c r="B1251" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="C1251" t="s">
         <v>393</v>
@@ -63412,7 +63466,7 @@
         <v>9029</v>
       </c>
       <c r="B1252" t="s">
-        <v>1363</v>
+        <v>1364</v>
       </c>
       <c r="C1252" t="s">
         <v>393</v>
@@ -63459,7 +63513,7 @@
         <v>9030</v>
       </c>
       <c r="B1253" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="C1253" t="s">
         <v>393</v>
@@ -63506,7 +63560,7 @@
         <v>9031</v>
       </c>
       <c r="B1254" t="s">
-        <v>1365</v>
+        <v>1366</v>
       </c>
       <c r="C1254" t="s">
         <v>393</v>
@@ -63553,7 +63607,7 @@
         <v>9032</v>
       </c>
       <c r="B1255" t="s">
-        <v>1366</v>
+        <v>1367</v>
       </c>
       <c r="C1255" t="s">
         <v>393</v>
@@ -63600,7 +63654,7 @@
         <v>9033</v>
       </c>
       <c r="B1256" t="s">
-        <v>1367</v>
+        <v>1368</v>
       </c>
       <c r="C1256" t="s">
         <v>393</v>
@@ -63647,7 +63701,7 @@
         <v>9034</v>
       </c>
       <c r="B1257" t="s">
-        <v>1368</v>
+        <v>1369</v>
       </c>
       <c r="C1257" t="s">
         <v>393</v>
@@ -63694,7 +63748,7 @@
         <v>9035</v>
       </c>
       <c r="B1258" t="s">
-        <v>1369</v>
+        <v>1370</v>
       </c>
       <c r="C1258" t="s">
         <v>393</v>
@@ -63741,7 +63795,7 @@
         <v>9036</v>
       </c>
       <c r="B1259" t="s">
-        <v>1370</v>
+        <v>1371</v>
       </c>
       <c r="C1259" t="s">
         <v>393</v>
@@ -63788,7 +63842,7 @@
         <v>9037</v>
       </c>
       <c r="B1260" t="s">
-        <v>1371</v>
+        <v>1372</v>
       </c>
       <c r="C1260" t="s">
         <v>393</v>
@@ -63835,7 +63889,7 @@
         <v>9038</v>
       </c>
       <c r="B1261" t="s">
-        <v>1372</v>
+        <v>1373</v>
       </c>
       <c r="C1261" t="s">
         <v>393</v>
@@ -63882,7 +63936,7 @@
         <v>9039</v>
       </c>
       <c r="B1262" t="s">
-        <v>1373</v>
+        <v>1374</v>
       </c>
       <c r="C1262" t="s">
         <v>427</v>
@@ -63929,7 +63983,7 @@
         <v>9040</v>
       </c>
       <c r="B1263" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="C1263" t="s">
         <v>393</v>
@@ -63976,7 +64030,7 @@
         <v>9041</v>
       </c>
       <c r="B1264" t="s">
-        <v>1375</v>
+        <v>1376</v>
       </c>
       <c r="C1264" t="s">
         <v>393</v>
@@ -64023,7 +64077,7 @@
         <v>9042</v>
       </c>
       <c r="B1265" t="s">
-        <v>1376</v>
+        <v>1377</v>
       </c>
       <c r="C1265" t="s">
         <v>393</v>
@@ -64070,7 +64124,7 @@
         <v>9043</v>
       </c>
       <c r="B1266" t="s">
-        <v>1377</v>
+        <v>1378</v>
       </c>
       <c r="C1266" t="s">
         <v>393</v>
@@ -64117,7 +64171,7 @@
         <v>9044</v>
       </c>
       <c r="B1267" t="s">
-        <v>1378</v>
+        <v>1379</v>
       </c>
       <c r="C1267" t="s">
         <v>393</v>
@@ -64164,7 +64218,7 @@
         <v>9045</v>
       </c>
       <c r="B1268" t="s">
-        <v>1379</v>
+        <v>1380</v>
       </c>
       <c r="C1268" t="s">
         <v>393</v>
@@ -64211,7 +64265,7 @@
         <v>9046</v>
       </c>
       <c r="B1269" t="s">
-        <v>1380</v>
+        <v>1381</v>
       </c>
       <c r="C1269" t="s">
         <v>393</v>
@@ -64258,7 +64312,7 @@
         <v>9047</v>
       </c>
       <c r="B1270" t="s">
-        <v>1381</v>
+        <v>1382</v>
       </c>
       <c r="C1270" t="s">
         <v>393</v>
@@ -64305,7 +64359,7 @@
         <v>9048</v>
       </c>
       <c r="B1271" t="s">
-        <v>1382</v>
+        <v>1383</v>
       </c>
       <c r="C1271" t="s">
         <v>393</v>
@@ -64352,7 +64406,7 @@
         <v>9049</v>
       </c>
       <c r="B1272" t="s">
-        <v>1383</v>
+        <v>1384</v>
       </c>
       <c r="C1272" t="s">
         <v>393</v>
@@ -64399,7 +64453,7 @@
         <v>9050</v>
       </c>
       <c r="B1273" t="s">
-        <v>1234</v>
+        <v>1235</v>
       </c>
       <c r="C1273" t="s">
         <v>393</v>
@@ -64446,7 +64500,7 @@
         <v>9051</v>
       </c>
       <c r="B1274" t="s">
-        <v>1384</v>
+        <v>1385</v>
       </c>
       <c r="C1274" t="s">
         <v>342</v>
@@ -64464,7 +64518,7 @@
         <v>0</v>
       </c>
       <c r="H1274" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="I1274" t="s">
         <v>19</v>
@@ -64493,7 +64547,7 @@
         <v>9052</v>
       </c>
       <c r="B1275" t="s">
-        <v>1385</v>
+        <v>1386</v>
       </c>
       <c r="C1275" t="s">
         <v>342</v>
@@ -64511,7 +64565,7 @@
         <v>0</v>
       </c>
       <c r="H1275" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="I1275" t="s">
         <v>19</v>
@@ -64540,7 +64594,7 @@
         <v>9053</v>
       </c>
       <c r="B1276" t="s">
-        <v>1386</v>
+        <v>1387</v>
       </c>
       <c r="C1276" t="s">
         <v>342</v>
@@ -64587,7 +64641,7 @@
         <v>9054</v>
       </c>
       <c r="B1277" t="s">
-        <v>1387</v>
+        <v>1388</v>
       </c>
       <c r="C1277" t="s">
         <v>342</v>
@@ -64634,7 +64688,7 @@
         <v>9055</v>
       </c>
       <c r="B1278" t="s">
-        <v>1388</v>
+        <v>1389</v>
       </c>
       <c r="C1278" t="s">
         <v>342</v>
@@ -64681,7 +64735,7 @@
         <v>9056</v>
       </c>
       <c r="B1279" t="s">
-        <v>1389</v>
+        <v>1390</v>
       </c>
       <c r="C1279" t="s">
         <v>342</v>
@@ -64728,7 +64782,7 @@
         <v>9057</v>
       </c>
       <c r="B1280" t="s">
-        <v>1390</v>
+        <v>1391</v>
       </c>
       <c r="C1280" t="s">
         <v>342</v>
@@ -64775,7 +64829,7 @@
         <v>9058</v>
       </c>
       <c r="B1281" t="s">
-        <v>1391</v>
+        <v>1392</v>
       </c>
       <c r="C1281" t="s">
         <v>342</v>
@@ -64822,7 +64876,7 @@
         <v>9060</v>
       </c>
       <c r="B1282" t="s">
-        <v>1392</v>
+        <v>1393</v>
       </c>
       <c r="C1282" t="s">
         <v>342</v>
@@ -64869,7 +64923,7 @@
         <v>9061</v>
       </c>
       <c r="B1283" t="s">
-        <v>1393</v>
+        <v>1394</v>
       </c>
       <c r="C1283" t="s">
         <v>342</v>
@@ -64916,7 +64970,7 @@
         <v>9062</v>
       </c>
       <c r="B1284" t="s">
-        <v>1394</v>
+        <v>1395</v>
       </c>
       <c r="C1284" t="s">
         <v>342</v>
@@ -64963,7 +65017,7 @@
         <v>9063</v>
       </c>
       <c r="B1285" t="s">
-        <v>1395</v>
+        <v>1396</v>
       </c>
       <c r="C1285" t="s">
         <v>342</v>
@@ -65010,7 +65064,7 @@
         <v>9064</v>
       </c>
       <c r="B1286" t="s">
-        <v>1396</v>
+        <v>1397</v>
       </c>
       <c r="C1286" t="s">
         <v>342</v>
@@ -65104,7 +65158,7 @@
         <v>9066</v>
       </c>
       <c r="B1288" t="s">
-        <v>1397</v>
+        <v>1398</v>
       </c>
       <c r="C1288" t="s">
         <v>464</v>
@@ -65151,7 +65205,7 @@
         <v>9067</v>
       </c>
       <c r="B1289" t="s">
-        <v>1398</v>
+        <v>1399</v>
       </c>
       <c r="C1289" t="s">
         <v>1163</v>
@@ -65198,7 +65252,7 @@
         <v>9068</v>
       </c>
       <c r="B1290" t="s">
-        <v>1399</v>
+        <v>1400</v>
       </c>
       <c r="C1290" t="s">
         <v>952</v>
@@ -65216,7 +65270,7 @@
         <v>0</v>
       </c>
       <c r="H1290" t="s">
-        <v>1400</v>
+        <v>1401</v>
       </c>
       <c r="I1290" t="s">
         <v>19</v>
@@ -65245,7 +65299,7 @@
         <v>9069</v>
       </c>
       <c r="B1291" t="s">
-        <v>1401</v>
+        <v>1402</v>
       </c>
       <c r="C1291" t="s">
         <v>464</v>
@@ -65292,7 +65346,7 @@
         <v>9070</v>
       </c>
       <c r="B1292" t="s">
-        <v>1402</v>
+        <v>1403</v>
       </c>
       <c r="C1292" t="s">
         <v>550</v>
@@ -65339,7 +65393,7 @@
         <v>9071</v>
       </c>
       <c r="B1293" t="s">
-        <v>1403</v>
+        <v>1404</v>
       </c>
       <c r="C1293" t="s">
         <v>497</v>
@@ -65357,7 +65411,7 @@
         <v>0</v>
       </c>
       <c r="H1293" t="s">
-        <v>1404</v>
+        <v>1405</v>
       </c>
       <c r="I1293" t="s">
         <v>19</v>
@@ -65404,7 +65458,7 @@
         <v>0</v>
       </c>
       <c r="H1294" t="s">
-        <v>1404</v>
+        <v>1405</v>
       </c>
       <c r="I1294" t="s">
         <v>19</v>
@@ -65433,7 +65487,7 @@
         <v>9073</v>
       </c>
       <c r="B1295" t="s">
-        <v>1405</v>
+        <v>1406</v>
       </c>
       <c r="C1295" t="s">
         <v>1163</v>
@@ -65451,7 +65505,7 @@
         <v>0</v>
       </c>
       <c r="H1295" t="s">
-        <v>1404</v>
+        <v>1405</v>
       </c>
       <c r="I1295" t="s">
         <v>19</v>
@@ -65480,7 +65534,7 @@
         <v>9074</v>
       </c>
       <c r="B1296" t="s">
-        <v>1406</v>
+        <v>1407</v>
       </c>
       <c r="C1296" t="s">
         <v>1163</v>
@@ -65498,7 +65552,7 @@
         <v>0</v>
       </c>
       <c r="H1296" t="s">
-        <v>1404</v>
+        <v>1405</v>
       </c>
       <c r="I1296" t="s">
         <v>19</v>
@@ -65527,7 +65581,7 @@
         <v>9075</v>
       </c>
       <c r="B1297" t="s">
-        <v>1407</v>
+        <v>1408</v>
       </c>
       <c r="C1297" t="s">
         <v>952</v>
@@ -65574,7 +65628,7 @@
         <v>9076</v>
       </c>
       <c r="B1298" t="s">
-        <v>1408</v>
+        <v>1409</v>
       </c>
       <c r="C1298" t="s">
         <v>537</v>
@@ -65621,7 +65675,7 @@
         <v>9077</v>
       </c>
       <c r="B1299" t="s">
-        <v>1409</v>
+        <v>1410</v>
       </c>
       <c r="C1299" t="s">
         <v>497</v>
@@ -65668,7 +65722,7 @@
         <v>9078</v>
       </c>
       <c r="B1300" t="s">
-        <v>1410</v>
+        <v>1411</v>
       </c>
       <c r="C1300" t="s">
         <v>749</v>
@@ -65715,7 +65769,7 @@
         <v>9079</v>
       </c>
       <c r="B1301" t="s">
-        <v>1411</v>
+        <v>1412</v>
       </c>
       <c r="C1301" t="s">
         <v>342</v>
@@ -65733,7 +65787,7 @@
         <v>0</v>
       </c>
       <c r="H1301" t="s">
-        <v>1412</v>
+        <v>1413</v>
       </c>
       <c r="I1301" t="s">
         <v>19</v>
@@ -65762,7 +65816,7 @@
         <v>9080</v>
       </c>
       <c r="B1302" t="s">
-        <v>1413</v>
+        <v>1414</v>
       </c>
       <c r="C1302" t="s">
         <v>749</v>
@@ -65809,7 +65863,7 @@
         <v>9081</v>
       </c>
       <c r="B1303" t="s">
-        <v>1414</v>
+        <v>1415</v>
       </c>
       <c r="C1303" t="s">
         <v>393</v>
@@ -65827,7 +65881,7 @@
         <v>0</v>
       </c>
       <c r="H1303" t="s">
-        <v>1400</v>
+        <v>1401</v>
       </c>
       <c r="I1303" t="s">
         <v>19</v>
@@ -65856,7 +65910,7 @@
         <v>9082</v>
       </c>
       <c r="B1304" t="s">
-        <v>1415</v>
+        <v>1416</v>
       </c>
       <c r="C1304" t="s">
         <v>342</v>
@@ -65874,7 +65928,7 @@
         <v>0</v>
       </c>
       <c r="H1304" t="s">
-        <v>1416</v>
+        <v>1417</v>
       </c>
       <c r="I1304" t="s">
         <v>19</v>
@@ -65910,9 +65964,358 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>1418</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1419</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1420</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1421</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2">
+        <v>8866</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1195</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1163</v>
+      </c>
+      <c r="D2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1422</v>
+      </c>
+      <c r="F2">
+        <v>200</v>
+      </c>
+      <c r="G2">
+        <v>200</v>
+      </c>
+      <c r="H2" t="s">
+        <v>1423</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1424</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3">
+        <v>83772</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1195</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1163</v>
+      </c>
+      <c r="D3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" t="s">
+        <v>1425</v>
+      </c>
+      <c r="F3">
+        <v>100</v>
+      </c>
+      <c r="G3">
+        <v>100</v>
+      </c>
+      <c r="H3" t="s">
+        <v>1423</v>
+      </c>
+      <c r="I3" t="s">
+        <v>1424</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4">
+        <v>83772</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1195</v>
+      </c>
+      <c r="C4" t="s">
+        <v>952</v>
+      </c>
+      <c r="D4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" t="s">
+        <v>1422</v>
+      </c>
+      <c r="F4">
+        <v>200</v>
+      </c>
+      <c r="G4">
+        <v>200</v>
+      </c>
+      <c r="H4" t="s">
+        <v>1423</v>
+      </c>
+      <c r="I4" t="s">
+        <v>1424</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5">
+        <v>83772</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1195</v>
+      </c>
+      <c r="C5" t="s">
+        <v>952</v>
+      </c>
+      <c r="D5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E5" t="s">
+        <v>1426</v>
+      </c>
+      <c r="F5" t="s">
+        <v>1427</v>
+      </c>
+      <c r="G5">
+        <v>150</v>
+      </c>
+      <c r="H5" t="s">
+        <v>1428</v>
+      </c>
+      <c r="I5" t="s">
+        <v>1424</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6">
+        <v>83772</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1195</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1163</v>
+      </c>
+      <c r="D6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" t="s">
+        <v>1429</v>
+      </c>
+      <c r="F6">
+        <v>6330</v>
+      </c>
+      <c r="G6">
+        <v>6330</v>
+      </c>
+      <c r="H6" t="s">
+        <v>1423</v>
+      </c>
+      <c r="I6" t="s">
+        <v>1430</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7">
+        <v>83772</v>
+      </c>
+      <c r="B7" t="s">
+        <v>1195</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1163</v>
+      </c>
+      <c r="D7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E7" t="s">
+        <v>1425</v>
+      </c>
+      <c r="F7">
+        <v>100</v>
+      </c>
+      <c r="G7">
+        <v>100</v>
+      </c>
+      <c r="H7" t="s">
+        <v>1423</v>
+      </c>
+      <c r="I7" t="s">
+        <v>1430</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8">
+        <v>83772</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1195</v>
+      </c>
+      <c r="C8" t="s">
+        <v>952</v>
+      </c>
+      <c r="D8" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" t="s">
+        <v>1431</v>
+      </c>
+      <c r="F8">
+        <v>50</v>
+      </c>
+      <c r="G8">
+        <v>50</v>
+      </c>
+      <c r="H8" t="s">
+        <v>1423</v>
+      </c>
+      <c r="I8" t="s">
+        <v>1430</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9">
+        <v>83772</v>
+      </c>
+      <c r="B9" t="s">
+        <v>1195</v>
+      </c>
+      <c r="C9" t="s">
+        <v>952</v>
+      </c>
+      <c r="D9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" t="s">
+        <v>1432</v>
+      </c>
+      <c r="F9">
+        <v>50</v>
+      </c>
+      <c r="G9">
+        <v>50</v>
+      </c>
+      <c r="H9" t="s">
+        <v>1423</v>
+      </c>
+      <c r="I9" t="s">
+        <v>1430</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10">
+        <v>83772</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1195</v>
+      </c>
+      <c r="C10" t="s">
+        <v>1163</v>
+      </c>
+      <c r="D10" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" t="s">
+        <v>1425</v>
+      </c>
+      <c r="F10">
+        <v>100</v>
+      </c>
+      <c r="G10">
+        <v>100</v>
+      </c>
+      <c r="H10" t="s">
+        <v>1433</v>
+      </c>
+      <c r="I10" t="s">
+        <v>1424</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11">
+        <v>8854</v>
+      </c>
+      <c r="B11" t="s">
+        <v>1177</v>
+      </c>
+      <c r="C11" t="s">
+        <v>952</v>
+      </c>
+      <c r="D11" t="s">
+        <v>339</v>
+      </c>
+      <c r="E11" t="s">
+        <v>1434</v>
+      </c>
+      <c r="F11">
+        <v>4000</v>
+      </c>
+      <c r="G11">
+        <v>4000</v>
+      </c>
+      <c r="H11" t="s">
+        <v>1433</v>
+      </c>
+      <c r="I11" t="s">
+        <v>1424</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12">
+        <v>8854</v>
+      </c>
+      <c r="B12" t="s">
+        <v>1177</v>
+      </c>
+      <c r="C12" t="s">
+        <v>952</v>
+      </c>
+      <c r="D12" t="s">
+        <v>339</v>
+      </c>
+      <c r="E12" t="s">
+        <v>1434</v>
+      </c>
+      <c r="F12">
+        <v>3000</v>
+      </c>
+      <c r="G12">
+        <v>3000</v>
+      </c>
+      <c r="H12" t="s">
+        <v>1433</v>
+      </c>
+      <c r="I12" t="s">
+        <v>1424</v>
+      </c>
+    </row>
+  </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>

</xml_diff>

<commit_message>
corrected the transaction table view
</commit_message>
<xml_diff>
--- a/backend/db/transfer/overall_data.xlsx
+++ b/backend/db/transfer/overall_data.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1442">
   <si>
     <t>admission</t>
   </si>
@@ -3511,817 +3511,838 @@
     <t>LKG</t>
   </si>
   <si>
+    <t>MOHAMMED RIFAZ M</t>
+  </si>
+  <si>
+    <t>HANIYA N</t>
+  </si>
+  <si>
+    <t>MOHAMMED ADYAN M Y</t>
+  </si>
+  <si>
+    <t>MYSHA FATHIMA M,</t>
+  </si>
+  <si>
+    <t>MOHAMMED M B</t>
+  </si>
+  <si>
+    <t>MOHAMED KHALID M</t>
+  </si>
+  <si>
+    <t>AYSHA LAIBA</t>
+  </si>
+  <si>
+    <t>AFEEKHA BANU S</t>
+  </si>
+  <si>
+    <t>SANVIKA P</t>
+  </si>
+  <si>
+    <t>MUHAMMAD AAKIF H</t>
+  </si>
+  <si>
+    <t>MOHAMMED SHAFWAAN</t>
+  </si>
+  <si>
+    <t>MOHAMED SHAHID AFRIDI S</t>
+  </si>
+  <si>
+    <t>ISHAQ AHAMED S</t>
+  </si>
+  <si>
+    <t>02/04/2023</t>
+  </si>
+  <si>
+    <t>AHAMED YASEEN AABID M</t>
+  </si>
+  <si>
+    <t>ZAFIR AHMAD A</t>
+  </si>
+  <si>
+    <t>05/04/2024</t>
+  </si>
+  <si>
+    <t>SAARA I</t>
+  </si>
+  <si>
+    <t>ABDULLAH</t>
+  </si>
+  <si>
+    <t>08/04/2024</t>
+  </si>
+  <si>
+    <t>RAIFA MARZOOKA R</t>
+  </si>
+  <si>
+    <t>17/04/2024</t>
+  </si>
+  <si>
+    <t>IFAAZ FAROOK T</t>
+  </si>
+  <si>
+    <t>15/04/2024</t>
+  </si>
+  <si>
+    <t>JAMAL HANIYA FATHIMA M</t>
+  </si>
+  <si>
+    <t>RAYYAN MAHMOUD M</t>
+  </si>
+  <si>
+    <t>MUHAMMAD TALHA</t>
+  </si>
+  <si>
+    <t>23/04/2024</t>
+  </si>
+  <si>
+    <t>ZAINAB UMAIZA A A</t>
+  </si>
+  <si>
+    <t>08/05/2024</t>
+  </si>
+  <si>
+    <t>MOHAMMAD ISHAAQ</t>
+  </si>
+  <si>
+    <t>MUHAMMAD RAYAAN M</t>
+  </si>
+  <si>
+    <t>MOHAMED HILMI M</t>
+  </si>
+  <si>
+    <t>AHAD MIKHAAIL H I</t>
+  </si>
+  <si>
+    <t>JAZEELA MAHJ M</t>
+  </si>
+  <si>
+    <t>MOHAMED HAMDAN M</t>
+  </si>
+  <si>
+    <t>AYAAN YUSUF A</t>
+  </si>
+  <si>
+    <t>ABDUL SHAHID S</t>
+  </si>
+  <si>
+    <t>MOHAMED NAWFAN M</t>
+  </si>
+  <si>
+    <t>UMAIMAH M J</t>
+  </si>
+  <si>
+    <t>MD SHAHID BASHA M</t>
+  </si>
+  <si>
+    <t>MUHAMMAD AAQIL</t>
+  </si>
+  <si>
+    <t>MOHAMED ISMAIL RAJA J</t>
+  </si>
+  <si>
+    <t>MOHAMMED RAFAN U</t>
+  </si>
+  <si>
+    <t>AHAMED IBRAHIM A M</t>
+  </si>
+  <si>
+    <t>FIZZA HADFAH S</t>
+  </si>
+  <si>
+    <t>ABBRAR HUSSAIN A</t>
+  </si>
+  <si>
+    <t>MOHAMED SAIFAN</t>
+  </si>
+  <si>
+    <t>MUHAMMAD ABDULLAH R</t>
+  </si>
+  <si>
+    <t>BASIM S K</t>
+  </si>
+  <si>
+    <t>MUHAMMAD ISHAQ</t>
+  </si>
+  <si>
+    <t>MOHAMMED UBAIDULLAH A</t>
+  </si>
+  <si>
+    <t>SYED ABUTHAHIR SHAYAAN I</t>
+  </si>
+  <si>
+    <t>ASMA RIFAYA M</t>
+  </si>
+  <si>
+    <t>03/04/2024</t>
+  </si>
+  <si>
+    <t>IFRAH MARIYAM M I</t>
+  </si>
+  <si>
+    <t>SAFNA J</t>
+  </si>
+  <si>
+    <t>NAWAZIYA FATHIMA I</t>
+  </si>
+  <si>
+    <t>06/05/2024</t>
+  </si>
+  <si>
+    <t>MOHAMMED HASHIM</t>
+  </si>
+  <si>
+    <t>SUHAINA S</t>
+  </si>
+  <si>
+    <t>MOHAMMED HAMZA M</t>
+  </si>
+  <si>
+    <t>MUHAMMAD</t>
+  </si>
+  <si>
+    <t>MD TAUSHIF</t>
+  </si>
+  <si>
+    <t>AAMEER HAMZA S</t>
+  </si>
+  <si>
+    <t>MUHAMMAD ZULQARNAIN M</t>
+  </si>
+  <si>
+    <t>SHAZIYA M</t>
+  </si>
+  <si>
+    <t>16/04/2024</t>
+  </si>
+  <si>
+    <t>SHIREEN NOWFIYA S</t>
+  </si>
+  <si>
+    <t>24/04/2024</t>
+  </si>
+  <si>
+    <t>SANA FATHIMA K</t>
+  </si>
+  <si>
+    <t>02/05/2024</t>
+  </si>
+  <si>
+    <t>MUHAMMAD ZIHAAN</t>
+  </si>
+  <si>
+    <t>ABDUL AZEEZ T</t>
+  </si>
+  <si>
+    <t>MOHAMED JASIM M</t>
+  </si>
+  <si>
+    <t>HAFSA UROOJ</t>
+  </si>
+  <si>
+    <t>KHAWLA FATHIMA</t>
+  </si>
+  <si>
+    <t>ABDUR RAHMAN N</t>
+  </si>
+  <si>
+    <t>BARAKATH NISHA</t>
+  </si>
+  <si>
+    <t>MOHAMMED ISMAIL</t>
+  </si>
+  <si>
+    <t>ARSHIYA BANU A</t>
+  </si>
+  <si>
+    <t>TAMIL MAGAN MUHAMMED IBRAHIM</t>
+  </si>
+  <si>
+    <t>RIDA RIFAET K</t>
+  </si>
+  <si>
+    <t>MOHAMED ABDUL KADIR</t>
+  </si>
+  <si>
+    <t>MUHAMMED FAAZIL M</t>
+  </si>
+  <si>
+    <t>FATHIMA SARA S</t>
+  </si>
+  <si>
+    <t>MOHAMED IBRAHIM AFAN</t>
+  </si>
+  <si>
+    <t>AYAAN KHAN</t>
+  </si>
+  <si>
+    <t>MUAZ N</t>
+  </si>
+  <si>
+    <t>ABU SHAHEED</t>
+  </si>
+  <si>
+    <t>MUHAMMAD FAIZ KHAN</t>
+  </si>
+  <si>
+    <t>MD SAAHIL BASHA M</t>
+  </si>
+  <si>
+    <t>MOHAMED AASIM AMBALAM</t>
+  </si>
+  <si>
+    <t>MD UBEDULA</t>
+  </si>
+  <si>
+    <t>MOHAMED</t>
+  </si>
+  <si>
+    <t>THAHSEENA</t>
+  </si>
+  <si>
+    <t>MOHAMED UMAR FAROOQ M</t>
+  </si>
+  <si>
+    <t>02/04/2024</t>
+  </si>
+  <si>
+    <t>ABDUL AHAD A</t>
+  </si>
+  <si>
+    <t>NASREEN M</t>
+  </si>
+  <si>
+    <t>IFRHA K</t>
+  </si>
+  <si>
+    <t>MOHAMMED AASHIQ D</t>
+  </si>
+  <si>
+    <t>INTHIHA FATHIMA</t>
+  </si>
+  <si>
+    <t>LIYA N</t>
+  </si>
+  <si>
+    <t>AFRAH A</t>
+  </si>
+  <si>
+    <t>BIBEKA SUNAR</t>
+  </si>
+  <si>
+    <t>YUMNAH</t>
+  </si>
+  <si>
+    <t>AALIYA SARA A</t>
+  </si>
+  <si>
+    <t>RAASHITHA PARVEEN A</t>
+  </si>
+  <si>
+    <t>MOHAMED FAAHIL N</t>
+  </si>
+  <si>
+    <t>MOHAMMED ISMAIL M</t>
+  </si>
+  <si>
+    <t>MUHAMMED FAZIS S</t>
+  </si>
+  <si>
+    <t>MOHAMMED YAMIN N</t>
+  </si>
+  <si>
+    <t>25/04/2024</t>
+  </si>
+  <si>
+    <t>ZIYA FATHIMA M S</t>
+  </si>
+  <si>
+    <t>KHALID MISHAL T M</t>
+  </si>
+  <si>
+    <t>MOHAMED ZAYAN N</t>
+  </si>
+  <si>
+    <t>SAFWAN J</t>
+  </si>
+  <si>
+    <t>MUHAMED SIKKANDAR M</t>
+  </si>
+  <si>
+    <t>MUHAMMED RAYYAN N</t>
+  </si>
+  <si>
+    <t>SAMRAH FATHIMA</t>
+  </si>
+  <si>
+    <t>JAFINA</t>
+  </si>
+  <si>
+    <t>MARYAM FAIHA</t>
+  </si>
+  <si>
+    <t>MOHAMMED AQIF BAIG N</t>
+  </si>
+  <si>
+    <t>MOHAMMED ZUBAIR B</t>
+  </si>
+  <si>
+    <t>HALITH IBRAHIM Y</t>
+  </si>
+  <si>
+    <t>RAHMATH NISA N</t>
+  </si>
+  <si>
+    <t>AYESHA MUVAFFEKA A</t>
+  </si>
+  <si>
+    <t>FAIZA FATHIMA J</t>
+  </si>
+  <si>
+    <t>MOHAMED SUHAIL A</t>
+  </si>
+  <si>
+    <t>SANA HUSNA M</t>
+  </si>
+  <si>
+    <t>ALEENA S</t>
+  </si>
+  <si>
+    <t>MOHAMMED FAZIL A</t>
+  </si>
+  <si>
+    <t>KATHIJA MEHAR R</t>
+  </si>
+  <si>
+    <t>MUHAMMED UWAIZ S</t>
+  </si>
+  <si>
+    <t>SANA FAIZIA T</t>
+  </si>
+  <si>
+    <t>SARA K</t>
+  </si>
+  <si>
+    <t>ARSHAD AHAMED A</t>
+  </si>
+  <si>
+    <t>ZUNAITH AHAMED R</t>
+  </si>
+  <si>
+    <t>ARSADDULLAH D</t>
+  </si>
+  <si>
+    <t>MARYAM SUMAIYA T</t>
+  </si>
+  <si>
+    <t>SARAFIYA BIVI S</t>
+  </si>
+  <si>
+    <t>IKRAM SHUBHAN S I</t>
+  </si>
+  <si>
+    <t>LYZA N</t>
+  </si>
+  <si>
+    <t>MOHAMED ASFAQ R</t>
+  </si>
+  <si>
+    <t>MOHAMMAD IKRAM I</t>
+  </si>
+  <si>
+    <t>BASIL HAMEEM A S</t>
+  </si>
+  <si>
+    <t>BASIQ HAMY A S</t>
+  </si>
+  <si>
+    <t>SARAH A</t>
+  </si>
+  <si>
+    <t>AFRAH FATHIMA B</t>
+  </si>
+  <si>
+    <t>THASLEEM C</t>
+  </si>
+  <si>
+    <t>MOHAMED HASHEEM D</t>
+  </si>
+  <si>
+    <t>MOHAMMED EBRAHIM M</t>
+  </si>
+  <si>
+    <t>MOHAMMED IRFAAN M</t>
+  </si>
+  <si>
+    <t>MUHAMMED FARHAAN S</t>
+  </si>
+  <si>
+    <t>MD FAIZAN</t>
+  </si>
+  <si>
+    <t>SYED DHANISH D</t>
+  </si>
+  <si>
+    <t>AFRIN KATHOON S</t>
+  </si>
+  <si>
+    <t>RIYA FATHIMA R</t>
+  </si>
+  <si>
+    <t>MURSHIDA FATHIMA K</t>
+  </si>
+  <si>
+    <t>AFERAN BANU A</t>
+  </si>
+  <si>
+    <t>SHARIFATUL INARA M</t>
+  </si>
+  <si>
+    <t>SANA NIHAR A</t>
+  </si>
+  <si>
+    <t>MOHAMMED IKRAASH SAIT A</t>
+  </si>
+  <si>
+    <t>MOHAMED NAFEES M I</t>
+  </si>
+  <si>
+    <t>MOHAMED FAYAS</t>
+  </si>
+  <si>
+    <t>MOHAMED FAWWAAZ S</t>
+  </si>
+  <si>
+    <t>THAKSHEEFA FATHIMA</t>
+  </si>
+  <si>
+    <t>MOHAMMAD RAIHAN F</t>
+  </si>
+  <si>
+    <t>MOHAMMAD AMAN ALI M</t>
+  </si>
+  <si>
+    <t>ARFAT ABU HAMZA</t>
+  </si>
+  <si>
+    <t>MUHAMMED AFFHAN S</t>
+  </si>
+  <si>
+    <t>MOHAMMED MUMAIYIZ S</t>
+  </si>
+  <si>
+    <t>26/04/2024</t>
+  </si>
+  <si>
+    <t>MOHAMMED ZUBAIR M S</t>
+  </si>
+  <si>
+    <t>AZRA FATHIMA V</t>
+  </si>
+  <si>
+    <t>UMAR FAROOQ Z</t>
+  </si>
+  <si>
+    <t>AFRAH BEGUM A</t>
+  </si>
+  <si>
+    <t>ADHIL HUSSAIN T Z</t>
+  </si>
+  <si>
+    <t>ABDUR RAAZIK I</t>
+  </si>
+  <si>
+    <t>ABDULLAH BILAL S</t>
+  </si>
+  <si>
+    <t>RAHAMATHULLAH S</t>
+  </si>
+  <si>
+    <t>AFIYA A</t>
+  </si>
+  <si>
+    <t>HAMDHAN SHARIFF R</t>
+  </si>
+  <si>
+    <t>SARA FATHIMA N</t>
+  </si>
+  <si>
+    <t>MUHAMMED RILWAN N</t>
+  </si>
+  <si>
+    <t>ZOYA RIFAET K</t>
+  </si>
+  <si>
+    <t>HAFIYA SULAIHAL S</t>
+  </si>
+  <si>
+    <t>ALTHAISEERA S</t>
+  </si>
+  <si>
+    <t>SANIYA ANJUM</t>
+  </si>
+  <si>
+    <t>MOHAMMED SAMEER S</t>
+  </si>
+  <si>
+    <t>MUHAMMAD HAMDAN A</t>
+  </si>
+  <si>
+    <t>THAHIRA</t>
+  </si>
+  <si>
+    <t>ALMIR A R</t>
+  </si>
+  <si>
+    <t>MOHAMMED SAFFICK S</t>
+  </si>
+  <si>
+    <t>MOHAMMED SITHICK S</t>
+  </si>
+  <si>
+    <t>MOHAMMED ASFI V</t>
+  </si>
+  <si>
+    <t>YAHYA AYYASH</t>
+  </si>
+  <si>
+    <t>ZAMRUL AMIR A</t>
+  </si>
+  <si>
+    <t>SHIFANA FATHIMA T</t>
+  </si>
+  <si>
+    <t>MUHAMMED SAFWAAN S B</t>
+  </si>
+  <si>
+    <t>ZULBIHAR AHMED</t>
+  </si>
+  <si>
+    <t>AHAMED IBRAHIM</t>
+  </si>
+  <si>
+    <t>MOHAMMED MUSTHAFA N</t>
+  </si>
+  <si>
+    <t>AISHA SIDDIQA T</t>
+  </si>
+  <si>
+    <t>ALIF KHAN A</t>
+  </si>
+  <si>
+    <t>IJASS AHAMED</t>
+  </si>
+  <si>
+    <t>MOHAMED WASIM KHAN N</t>
+  </si>
+  <si>
+    <t>FATHIMA NABEELA P</t>
+  </si>
+  <si>
+    <t>ISMAIL M</t>
+  </si>
+  <si>
+    <t>MOHAMMAD RIYAZ</t>
+  </si>
+  <si>
+    <t>ABDUR RAHMAN S</t>
+  </si>
+  <si>
+    <t>MOHAMED ABEER KHAN M A</t>
+  </si>
+  <si>
+    <t>ABRAR AHAMED A</t>
+  </si>
+  <si>
+    <t>ASHIQ AHMED A</t>
+  </si>
+  <si>
+    <t>MOHIDEEN HAFEEZ K S</t>
+  </si>
+  <si>
+    <t>MUSKAAN S</t>
+  </si>
+  <si>
+    <t>MOHAMED ASRAR</t>
+  </si>
+  <si>
+    <t>AHAMED SAAD N</t>
+  </si>
+  <si>
+    <t>MOHAMMED HAATHIM</t>
+  </si>
+  <si>
+    <t>SAMEENA FATHIN S K</t>
+  </si>
+  <si>
+    <t>MOHAMED NAZAR FAYAZ A</t>
+  </si>
+  <si>
+    <t>SHAMIR AHAMED S</t>
+  </si>
+  <si>
+    <t>ZAHIA FATHIMA A A</t>
+  </si>
+  <si>
+    <t>SEYED AFIQ</t>
+  </si>
+  <si>
+    <t>MOHAMED AQUIL HUSSAIN</t>
+  </si>
+  <si>
+    <t>FAAIQUA MAHASIN S B</t>
+  </si>
+  <si>
+    <t>AYAAN AHMED U</t>
+  </si>
+  <si>
+    <t>MUHAMMAD IRSHAAD Y</t>
+  </si>
+  <si>
+    <t>MOHAMED SHAHID N</t>
+  </si>
+  <si>
+    <t>MOHAMED ALI S A</t>
+  </si>
+  <si>
+    <t>ALISHA A</t>
+  </si>
+  <si>
+    <t>MOHAMED NAVFAL N</t>
+  </si>
+  <si>
+    <t>THOUFIQ KHAN S</t>
+  </si>
+  <si>
+    <t>MUHAMMAD ARMAAN F</t>
+  </si>
+  <si>
+    <t>MAFAAZ M</t>
+  </si>
+  <si>
+    <t>03/07/2024</t>
+  </si>
+  <si>
+    <t>AASMIN KHATOON</t>
+  </si>
+  <si>
+    <t>FAIJAL SAH</t>
+  </si>
+  <si>
+    <t>MAHDI M</t>
+  </si>
+  <si>
+    <t>09/07/2024</t>
+  </si>
+  <si>
+    <t>HAIDAR ALI SAH</t>
+  </si>
+  <si>
+    <t>GAUSAIYA KHATOON</t>
+  </si>
+  <si>
+    <t>SEHERIN KHAN</t>
+  </si>
+  <si>
+    <t>TAIBA KHATUN</t>
+  </si>
+  <si>
+    <t>MOHAMED AFFAN KHAN M A</t>
+  </si>
+  <si>
+    <t>FATHIMA MAHIRA K</t>
+  </si>
+  <si>
+    <t>HIBA</t>
+  </si>
+  <si>
+    <t>01/08/2024</t>
+  </si>
+  <si>
+    <t>SAYMA PARVEEN</t>
+  </si>
+  <si>
+    <t>SANA FATHIMA M</t>
+  </si>
+  <si>
+    <t>MOHAMED THARIC M</t>
+  </si>
+  <si>
+    <t>22/08/2024</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>amount</t>
+  </si>
+  <si>
+    <t>total</t>
+  </si>
+  <si>
+    <t>mode</t>
+  </si>
+  <si>
+    <t>new admission application</t>
+  </si>
+  <si>
+    <t>04/02/2025</t>
+  </si>
+  <si>
+    <t>cash</t>
+  </si>
+  <si>
+    <t>id card</t>
+  </si>
+  <si>
+    <t>belt,id card</t>
+  </si>
+  <si>
+    <t>50,100</t>
+  </si>
+  <si>
+    <t>05/02/2025</t>
+  </si>
+  <si>
+    <t>term iii</t>
+  </si>
+  <si>
+    <t>cheque_online</t>
+  </si>
+  <si>
+    <t>bonafide certificate</t>
+  </si>
+  <si>
+    <t>belt</t>
+  </si>
+  <si>
+    <t>06/02/2025</t>
+  </si>
+  <si>
+    <t>term ii</t>
+  </si>
+  <si>
     <t>09/02/2025</t>
   </si>
   <si>
-    <t>MOHAMMED RIFAZ M</t>
-  </si>
-  <si>
-    <t>HANIYA N</t>
-  </si>
-  <si>
-    <t>MOHAMMED ADYAN M Y</t>
-  </si>
-  <si>
-    <t>MYSHA FATHIMA M,</t>
-  </si>
-  <si>
-    <t>MOHAMMED M B</t>
-  </si>
-  <si>
-    <t>MOHAMED KHALID M</t>
-  </si>
-  <si>
-    <t>AYSHA LAIBA</t>
-  </si>
-  <si>
-    <t>AFEEKHA BANU S</t>
-  </si>
-  <si>
-    <t>SANVIKA P</t>
-  </si>
-  <si>
-    <t>MUHAMMAD AAKIF H</t>
-  </si>
-  <si>
-    <t>MOHAMMED SHAFWAAN</t>
-  </si>
-  <si>
-    <t>MOHAMED SHAHID AFRIDI S</t>
-  </si>
-  <si>
-    <t>ISHAQ AHAMED S</t>
-  </si>
-  <si>
-    <t>02/04/2023</t>
-  </si>
-  <si>
-    <t>AHAMED YASEEN AABID M</t>
-  </si>
-  <si>
-    <t>ZAFIR AHMAD A</t>
-  </si>
-  <si>
-    <t>05/04/2024</t>
-  </si>
-  <si>
-    <t>SAARA I</t>
-  </si>
-  <si>
-    <t>ABDULLAH</t>
-  </si>
-  <si>
-    <t>08/04/2024</t>
-  </si>
-  <si>
-    <t>RAIFA MARZOOKA R</t>
-  </si>
-  <si>
-    <t>17/04/2024</t>
-  </si>
-  <si>
-    <t>IFAAZ FAROOK T</t>
-  </si>
-  <si>
-    <t>15/04/2024</t>
-  </si>
-  <si>
-    <t>JAMAL HANIYA FATHIMA M</t>
-  </si>
-  <si>
-    <t>RAYYAN MAHMOUD M</t>
-  </si>
-  <si>
-    <t>MUHAMMAD TALHA</t>
-  </si>
-  <si>
-    <t>23/04/2024</t>
-  </si>
-  <si>
-    <t>ZAINAB UMAIZA A A</t>
-  </si>
-  <si>
-    <t>08/05/2024</t>
-  </si>
-  <si>
-    <t>MOHAMMAD ISHAAQ</t>
-  </si>
-  <si>
-    <t>MUHAMMAD RAYAAN M</t>
-  </si>
-  <si>
-    <t>MOHAMED HILMI M</t>
-  </si>
-  <si>
-    <t>AHAD MIKHAAIL H I</t>
-  </si>
-  <si>
-    <t>JAZEELA MAHJ M</t>
-  </si>
-  <si>
-    <t>MOHAMED HAMDAN M</t>
-  </si>
-  <si>
-    <t>AYAAN YUSUF A</t>
-  </si>
-  <si>
-    <t>ABDUL SHAHID S</t>
-  </si>
-  <si>
-    <t>MOHAMED NAWFAN M</t>
-  </si>
-  <si>
-    <t>UMAIMAH M J</t>
-  </si>
-  <si>
-    <t>MD SHAHID BASHA M</t>
-  </si>
-  <si>
-    <t>MUHAMMAD AAQIL</t>
-  </si>
-  <si>
-    <t>MOHAMED ISMAIL RAJA J</t>
-  </si>
-  <si>
-    <t>MOHAMMED RAFAN U</t>
-  </si>
-  <si>
-    <t>AHAMED IBRAHIM A M</t>
-  </si>
-  <si>
-    <t>FIZZA HADFAH S</t>
-  </si>
-  <si>
-    <t>ABBRAR HUSSAIN A</t>
-  </si>
-  <si>
-    <t>MOHAMED SAIFAN</t>
-  </si>
-  <si>
-    <t>MUHAMMAD ABDULLAH R</t>
-  </si>
-  <si>
-    <t>BASIM S K</t>
-  </si>
-  <si>
-    <t>MUHAMMAD ISHAQ</t>
-  </si>
-  <si>
-    <t>MOHAMMED UBAIDULLAH A</t>
-  </si>
-  <si>
-    <t>SYED ABUTHAHIR SHAYAAN I</t>
-  </si>
-  <si>
-    <t>ASMA RIFAYA M</t>
-  </si>
-  <si>
-    <t>03/04/2024</t>
-  </si>
-  <si>
-    <t>IFRAH MARIYAM M I</t>
-  </si>
-  <si>
-    <t>SAFNA J</t>
-  </si>
-  <si>
-    <t>NAWAZIYA FATHIMA I</t>
-  </si>
-  <si>
-    <t>06/05/2024</t>
-  </si>
-  <si>
-    <t>MOHAMMED HASHIM</t>
-  </si>
-  <si>
-    <t>SUHAINA S</t>
-  </si>
-  <si>
-    <t>MOHAMMED HAMZA M</t>
-  </si>
-  <si>
-    <t>MUHAMMAD</t>
-  </si>
-  <si>
-    <t>MD TAUSHIF</t>
-  </si>
-  <si>
-    <t>AAMEER HAMZA S</t>
-  </si>
-  <si>
-    <t>MUHAMMAD ZULQARNAIN M</t>
-  </si>
-  <si>
-    <t>SHAZIYA M</t>
-  </si>
-  <si>
-    <t>16/04/2024</t>
-  </si>
-  <si>
-    <t>SHIREEN NOWFIYA S</t>
-  </si>
-  <si>
-    <t>24/04/2024</t>
-  </si>
-  <si>
-    <t>SANA FATHIMA K</t>
-  </si>
-  <si>
-    <t>02/05/2024</t>
-  </si>
-  <si>
-    <t>MUHAMMAD ZIHAAN</t>
-  </si>
-  <si>
-    <t>ABDUL AZEEZ T</t>
-  </si>
-  <si>
-    <t>MOHAMED JASIM M</t>
-  </si>
-  <si>
-    <t>HAFSA UROOJ</t>
-  </si>
-  <si>
-    <t>KHAWLA FATHIMA</t>
-  </si>
-  <si>
-    <t>ABDUR RAHMAN N</t>
-  </si>
-  <si>
-    <t>BARAKATH NISHA</t>
-  </si>
-  <si>
-    <t>MOHAMMED ISMAIL</t>
-  </si>
-  <si>
-    <t>ARSHIYA BANU A</t>
-  </si>
-  <si>
-    <t>TAMIL MAGAN MUHAMMED IBRAHIM</t>
-  </si>
-  <si>
-    <t>RIDA RIFAET K</t>
-  </si>
-  <si>
-    <t>MOHAMED ABDUL KADIR</t>
-  </si>
-  <si>
-    <t>MUHAMMED FAAZIL M</t>
-  </si>
-  <si>
-    <t>FATHIMA SARA S</t>
-  </si>
-  <si>
-    <t>MOHAMED IBRAHIM AFAN</t>
-  </si>
-  <si>
-    <t>AYAAN KHAN</t>
-  </si>
-  <si>
-    <t>MUAZ N</t>
-  </si>
-  <si>
-    <t>ABU SHAHEED</t>
-  </si>
-  <si>
-    <t>MUHAMMAD FAIZ KHAN</t>
-  </si>
-  <si>
-    <t>MD SAAHIL BASHA M</t>
-  </si>
-  <si>
-    <t>MOHAMED AASIM AMBALAM</t>
-  </si>
-  <si>
-    <t>MD UBEDULA</t>
-  </si>
-  <si>
-    <t>MOHAMED</t>
-  </si>
-  <si>
-    <t>THAHSEENA</t>
-  </si>
-  <si>
-    <t>MOHAMED UMAR FAROOQ M</t>
-  </si>
-  <si>
-    <t>02/04/2024</t>
-  </si>
-  <si>
-    <t>ABDUL AHAD A</t>
-  </si>
-  <si>
-    <t>NASREEN M</t>
-  </si>
-  <si>
-    <t>IFRHA K</t>
-  </si>
-  <si>
-    <t>MOHAMMED AASHIQ D</t>
-  </si>
-  <si>
-    <t>INTHIHA FATHIMA</t>
-  </si>
-  <si>
-    <t>LIYA N</t>
-  </si>
-  <si>
-    <t>AFRAH A</t>
-  </si>
-  <si>
-    <t>BIBEKA SUNAR</t>
-  </si>
-  <si>
-    <t>YUMNAH</t>
-  </si>
-  <si>
-    <t>AALIYA SARA A</t>
-  </si>
-  <si>
-    <t>RAASHITHA PARVEEN A</t>
-  </si>
-  <si>
-    <t>MOHAMED FAAHIL N</t>
-  </si>
-  <si>
-    <t>MOHAMMED ISMAIL M</t>
-  </si>
-  <si>
-    <t>MUHAMMED FAZIS S</t>
-  </si>
-  <si>
-    <t>MOHAMMED YAMIN N</t>
-  </si>
-  <si>
-    <t>25/04/2024</t>
-  </si>
-  <si>
-    <t>ZIYA FATHIMA M S</t>
-  </si>
-  <si>
-    <t>KHALID MISHAL T M</t>
-  </si>
-  <si>
-    <t>MOHAMED ZAYAN N</t>
-  </si>
-  <si>
-    <t>SAFWAN J</t>
-  </si>
-  <si>
-    <t>MUHAMED SIKKANDAR M</t>
-  </si>
-  <si>
-    <t>MUHAMMED RAYYAN N</t>
-  </si>
-  <si>
-    <t>SAMRAH FATHIMA</t>
-  </si>
-  <si>
-    <t>JAFINA</t>
-  </si>
-  <si>
-    <t>MARYAM FAIHA</t>
-  </si>
-  <si>
-    <t>MOHAMMED AQIF BAIG N</t>
-  </si>
-  <si>
-    <t>MOHAMMED ZUBAIR B</t>
-  </si>
-  <si>
-    <t>HALITH IBRAHIM Y</t>
-  </si>
-  <si>
-    <t>RAHMATH NISA N</t>
-  </si>
-  <si>
-    <t>AYESHA MUVAFFEKA A</t>
-  </si>
-  <si>
-    <t>FAIZA FATHIMA J</t>
-  </si>
-  <si>
-    <t>MOHAMED SUHAIL A</t>
-  </si>
-  <si>
-    <t>SANA HUSNA M</t>
-  </si>
-  <si>
-    <t>ALEENA S</t>
-  </si>
-  <si>
-    <t>MOHAMMED FAZIL A</t>
-  </si>
-  <si>
-    <t>KATHIJA MEHAR R</t>
-  </si>
-  <si>
-    <t>MUHAMMED UWAIZ S</t>
-  </si>
-  <si>
-    <t>SANA FAIZIA T</t>
-  </si>
-  <si>
-    <t>SARA K</t>
-  </si>
-  <si>
-    <t>ARSHAD AHAMED A</t>
-  </si>
-  <si>
-    <t>ZUNAITH AHAMED R</t>
-  </si>
-  <si>
-    <t>ARSADDULLAH D</t>
-  </si>
-  <si>
-    <t>MARYAM SUMAIYA T</t>
-  </si>
-  <si>
-    <t>SARAFIYA BIVI S</t>
-  </si>
-  <si>
-    <t>IKRAM SHUBHAN S I</t>
-  </si>
-  <si>
-    <t>LYZA N</t>
-  </si>
-  <si>
-    <t>MOHAMED ASFAQ R</t>
-  </si>
-  <si>
-    <t>MOHAMMAD IKRAM I</t>
-  </si>
-  <si>
-    <t>BASIL HAMEEM A S</t>
-  </si>
-  <si>
-    <t>BASIQ HAMY A S</t>
-  </si>
-  <si>
-    <t>SARAH A</t>
-  </si>
-  <si>
-    <t>AFRAH FATHIMA B</t>
-  </si>
-  <si>
-    <t>THASLEEM C</t>
-  </si>
-  <si>
-    <t>MOHAMED HASHEEM D</t>
-  </si>
-  <si>
-    <t>MOHAMMED EBRAHIM M</t>
-  </si>
-  <si>
-    <t>MOHAMMED IRFAAN M</t>
-  </si>
-  <si>
-    <t>MUHAMMED FARHAAN S</t>
-  </si>
-  <si>
-    <t>MD FAIZAN</t>
-  </si>
-  <si>
-    <t>SYED DHANISH D</t>
-  </si>
-  <si>
-    <t>AFRIN KATHOON S</t>
-  </si>
-  <si>
-    <t>RIYA FATHIMA R</t>
-  </si>
-  <si>
-    <t>MURSHIDA FATHIMA K</t>
-  </si>
-  <si>
-    <t>AFERAN BANU A</t>
-  </si>
-  <si>
-    <t>SHARIFATUL INARA M</t>
-  </si>
-  <si>
-    <t>SANA NIHAR A</t>
-  </si>
-  <si>
-    <t>MOHAMMED IKRAASH SAIT A</t>
-  </si>
-  <si>
-    <t>MOHAMED NAFEES M I</t>
-  </si>
-  <si>
-    <t>MOHAMED FAYAS</t>
-  </si>
-  <si>
-    <t>MOHAMED FAWWAAZ S</t>
-  </si>
-  <si>
-    <t>THAKSHEEFA FATHIMA</t>
-  </si>
-  <si>
-    <t>MOHAMMAD RAIHAN F</t>
-  </si>
-  <si>
-    <t>MOHAMMAD AMAN ALI M</t>
-  </si>
-  <si>
-    <t>ARFAT ABU HAMZA</t>
-  </si>
-  <si>
-    <t>MUHAMMED AFFHAN S</t>
-  </si>
-  <si>
-    <t>MOHAMMED MUMAIYIZ S</t>
-  </si>
-  <si>
-    <t>26/04/2024</t>
-  </si>
-  <si>
-    <t>MOHAMMED ZUBAIR M S</t>
-  </si>
-  <si>
-    <t>AZRA FATHIMA V</t>
-  </si>
-  <si>
-    <t>UMAR FAROOQ Z</t>
-  </si>
-  <si>
-    <t>AFRAH BEGUM A</t>
-  </si>
-  <si>
-    <t>ADHIL HUSSAIN T Z</t>
-  </si>
-  <si>
-    <t>ABDUR RAAZIK I</t>
-  </si>
-  <si>
-    <t>ABDULLAH BILAL S</t>
-  </si>
-  <si>
-    <t>RAHAMATHULLAH S</t>
-  </si>
-  <si>
-    <t>AFIYA A</t>
-  </si>
-  <si>
-    <t>HAMDHAN SHARIFF R</t>
-  </si>
-  <si>
-    <t>SARA FATHIMA N</t>
-  </si>
-  <si>
-    <t>MUHAMMED RILWAN N</t>
-  </si>
-  <si>
-    <t>ZOYA RIFAET K</t>
-  </si>
-  <si>
-    <t>HAFIYA SULAIHAL S</t>
-  </si>
-  <si>
-    <t>ALTHAISEERA S</t>
-  </si>
-  <si>
-    <t>SANIYA ANJUM</t>
-  </si>
-  <si>
-    <t>MOHAMMED SAMEER S</t>
-  </si>
-  <si>
-    <t>MUHAMMAD HAMDAN A</t>
-  </si>
-  <si>
-    <t>THAHIRA</t>
-  </si>
-  <si>
-    <t>ALMIR A R</t>
-  </si>
-  <si>
-    <t>MOHAMMED SAFFICK S</t>
-  </si>
-  <si>
-    <t>MOHAMMED SITHICK S</t>
-  </si>
-  <si>
-    <t>MOHAMMED ASFI V</t>
-  </si>
-  <si>
-    <t>YAHYA AYYASH</t>
-  </si>
-  <si>
-    <t>ZAMRUL AMIR A</t>
-  </si>
-  <si>
-    <t>SHIFANA FATHIMA T</t>
-  </si>
-  <si>
-    <t>MUHAMMED SAFWAAN S B</t>
-  </si>
-  <si>
-    <t>ZULBIHAR AHMED</t>
-  </si>
-  <si>
-    <t>AHAMED IBRAHIM</t>
-  </si>
-  <si>
-    <t>MOHAMMED MUSTHAFA N</t>
-  </si>
-  <si>
-    <t>AISHA SIDDIQA T</t>
-  </si>
-  <si>
-    <t>ALIF KHAN A</t>
-  </si>
-  <si>
-    <t>IJASS AHAMED</t>
-  </si>
-  <si>
-    <t>MOHAMED WASIM KHAN N</t>
-  </si>
-  <si>
-    <t>FATHIMA NABEELA P</t>
-  </si>
-  <si>
-    <t>ISMAIL M</t>
-  </si>
-  <si>
-    <t>MOHAMMAD RIYAZ</t>
-  </si>
-  <si>
-    <t>ABDUR RAHMAN S</t>
-  </si>
-  <si>
-    <t>MOHAMED ABEER KHAN M A</t>
-  </si>
-  <si>
-    <t>ABRAR AHAMED A</t>
-  </si>
-  <si>
-    <t>ASHIQ AHMED A</t>
-  </si>
-  <si>
-    <t>MOHIDEEN HAFEEZ K S</t>
-  </si>
-  <si>
-    <t>MUSKAAN S</t>
-  </si>
-  <si>
-    <t>MOHAMED ASRAR</t>
-  </si>
-  <si>
-    <t>AHAMED SAAD N</t>
-  </si>
-  <si>
-    <t>MOHAMMED HAATHIM</t>
-  </si>
-  <si>
-    <t>SAMEENA FATHIN S K</t>
-  </si>
-  <si>
-    <t>MOHAMED NAZAR FAYAZ A</t>
-  </si>
-  <si>
-    <t>SHAMIR AHAMED S</t>
-  </si>
-  <si>
-    <t>ZAHIA FATHIMA A A</t>
-  </si>
-  <si>
-    <t>SEYED AFIQ</t>
-  </si>
-  <si>
-    <t>MOHAMED AQUIL HUSSAIN</t>
-  </si>
-  <si>
-    <t>FAAIQUA MAHASIN S B</t>
-  </si>
-  <si>
-    <t>AYAAN AHMED U</t>
-  </si>
-  <si>
-    <t>MUHAMMAD IRSHAAD Y</t>
-  </si>
-  <si>
-    <t>MOHAMED SHAHID N</t>
-  </si>
-  <si>
-    <t>MOHAMED ALI S A</t>
-  </si>
-  <si>
-    <t>ALISHA A</t>
-  </si>
-  <si>
-    <t>MOHAMED NAVFAL N</t>
-  </si>
-  <si>
-    <t>THOUFIQ KHAN S</t>
-  </si>
-  <si>
-    <t>MUHAMMAD ARMAAN F</t>
-  </si>
-  <si>
-    <t>MAFAAZ M</t>
-  </si>
-  <si>
-    <t>03/07/2024</t>
-  </si>
-  <si>
-    <t>AASMIN KHATOON</t>
-  </si>
-  <si>
-    <t>FAIJAL SAH</t>
-  </si>
-  <si>
-    <t>MAHDI M</t>
-  </si>
-  <si>
-    <t>09/07/2024</t>
-  </si>
-  <si>
-    <t>HAIDAR ALI SAH</t>
-  </si>
-  <si>
-    <t>GAUSAIYA KHATOON</t>
-  </si>
-  <si>
-    <t>SEHERIN KHAN</t>
-  </si>
-  <si>
-    <t>TAIBA KHATUN</t>
-  </si>
-  <si>
-    <t>MOHAMED AFFAN KHAN M A</t>
-  </si>
-  <si>
-    <t>FATHIMA MAHIRA K</t>
-  </si>
-  <si>
-    <t>HIBA</t>
-  </si>
-  <si>
-    <t>01/08/2024</t>
-  </si>
-  <si>
-    <t>SAYMA PARVEEN</t>
-  </si>
-  <si>
-    <t>SANA FATHIMA M</t>
-  </si>
-  <si>
-    <t>MOHAMED THARIC M</t>
-  </si>
-  <si>
-    <t>22/08/2024</t>
-  </si>
-  <si>
-    <t>type</t>
-  </si>
-  <si>
-    <t>amount</t>
-  </si>
-  <si>
-    <t>total</t>
-  </si>
-  <si>
-    <t>mode</t>
-  </si>
-  <si>
-    <t>new admission application</t>
-  </si>
-  <si>
-    <t>04/02/2025</t>
-  </si>
-  <si>
-    <t>cash</t>
-  </si>
-  <si>
-    <t>id card</t>
-  </si>
-  <si>
-    <t>belt,id card</t>
-  </si>
-  <si>
-    <t>50,100</t>
-  </si>
-  <si>
-    <t>05/02/2025</t>
-  </si>
-  <si>
-    <t>term iii</t>
-  </si>
-  <si>
-    <t>cheque_online</t>
-  </si>
-  <si>
-    <t>bonafide certificate</t>
-  </si>
-  <si>
-    <t>belt</t>
-  </si>
-  <si>
-    <t>06/02/2025</t>
-  </si>
-  <si>
-    <t>term ii</t>
+    <t>HIBAH FATIMA</t>
+  </si>
+  <si>
+    <t>id card,new admission application</t>
+  </si>
+  <si>
+    <t>100,200</t>
+  </si>
+  <si>
+    <t>report card</t>
+  </si>
+  <si>
+    <t>15/02/2025</t>
+  </si>
+  <si>
+    <t>term i</t>
+  </si>
+  <si>
+    <t>19/03/2025</t>
   </si>
 </sst>
 </file>
@@ -54648,7 +54669,7 @@
         <v>0</v>
       </c>
       <c r="H1064" t="s">
-        <v>1164</v>
+        <v>44</v>
       </c>
       <c r="I1064" t="s">
         <v>462</v>
@@ -54657,19 +54678,19 @@
         <v>20330</v>
       </c>
       <c r="K1064">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="L1064">
         <v>0</v>
       </c>
       <c r="M1064">
-        <v>23330</v>
+        <v>20330</v>
       </c>
       <c r="N1064">
         <v>20330</v>
       </c>
       <c r="O1064">
-        <v>3000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1065" spans="1:15">
@@ -54677,7 +54698,7 @@
         <v>8840</v>
       </c>
       <c r="B1065" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="C1065" t="s">
         <v>1163</v>
@@ -54724,7 +54745,7 @@
         <v>8841</v>
       </c>
       <c r="B1066" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="C1066" t="s">
         <v>1163</v>
@@ -54771,7 +54792,7 @@
         <v>8842</v>
       </c>
       <c r="B1067" t="s">
-        <v>1167</v>
+        <v>1166</v>
       </c>
       <c r="C1067" t="s">
         <v>1163</v>
@@ -54818,7 +54839,7 @@
         <v>8843</v>
       </c>
       <c r="B1068" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="C1068" t="s">
         <v>1163</v>
@@ -54865,7 +54886,7 @@
         <v>8844</v>
       </c>
       <c r="B1069" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="C1069" t="s">
         <v>1163</v>
@@ -54959,7 +54980,7 @@
         <v>8846</v>
       </c>
       <c r="B1071" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
       <c r="C1071" t="s">
         <v>1163</v>
@@ -55006,7 +55027,7 @@
         <v>8847</v>
       </c>
       <c r="B1072" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
       <c r="C1072" t="s">
         <v>1163</v>
@@ -55053,7 +55074,7 @@
         <v>8848</v>
       </c>
       <c r="B1073" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
       <c r="C1073" t="s">
         <v>1163</v>
@@ -55100,7 +55121,7 @@
         <v>8849</v>
       </c>
       <c r="B1074" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C1074" t="s">
         <v>1163</v>
@@ -55147,7 +55168,7 @@
         <v>8850</v>
       </c>
       <c r="B1075" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="C1075" t="s">
         <v>1163</v>
@@ -55194,7 +55215,7 @@
         <v>8851</v>
       </c>
       <c r="B1076" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="C1076" t="s">
         <v>1163</v>
@@ -55241,7 +55262,7 @@
         <v>8852</v>
       </c>
       <c r="B1077" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="C1077" t="s">
         <v>1163</v>
@@ -55288,7 +55309,7 @@
         <v>8854</v>
       </c>
       <c r="B1078" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="C1078" t="s">
         <v>1163</v>
@@ -55306,7 +55327,7 @@
         <v>0</v>
       </c>
       <c r="H1078" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="I1078" t="s">
         <v>19</v>
@@ -55335,7 +55356,7 @@
         <v>8855</v>
       </c>
       <c r="B1079" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="C1079" t="s">
         <v>1163</v>
@@ -55353,7 +55374,7 @@
         <v>0</v>
       </c>
       <c r="H1079" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="I1079" t="s">
         <v>19</v>
@@ -55382,7 +55403,7 @@
         <v>8857</v>
       </c>
       <c r="B1080" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
       <c r="C1080" t="s">
         <v>1163</v>
@@ -55400,7 +55421,7 @@
         <v>0</v>
       </c>
       <c r="H1080" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="I1080" t="s">
         <v>19</v>
@@ -55429,7 +55450,7 @@
         <v>8858</v>
       </c>
       <c r="B1081" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
       <c r="C1081" t="s">
         <v>1163</v>
@@ -55447,7 +55468,7 @@
         <v>0</v>
       </c>
       <c r="H1081" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="I1081" t="s">
         <v>19</v>
@@ -55476,7 +55497,7 @@
         <v>8859</v>
       </c>
       <c r="B1082" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="C1082" t="s">
         <v>1163</v>
@@ -55494,7 +55515,7 @@
         <v>0</v>
       </c>
       <c r="H1082" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
       <c r="I1082" t="s">
         <v>19</v>
@@ -55523,7 +55544,7 @@
         <v>8860</v>
       </c>
       <c r="B1083" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="C1083" t="s">
         <v>1163</v>
@@ -55541,7 +55562,7 @@
         <v>0</v>
       </c>
       <c r="H1083" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="I1083" t="s">
         <v>19</v>
@@ -55570,7 +55591,7 @@
         <v>8861</v>
       </c>
       <c r="B1084" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="C1084" t="s">
         <v>1163</v>
@@ -55588,7 +55609,7 @@
         <v>0</v>
       </c>
       <c r="H1084" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="I1084" t="s">
         <v>19</v>
@@ -55617,7 +55638,7 @@
         <v>8862</v>
       </c>
       <c r="B1085" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="C1085" t="s">
         <v>1163</v>
@@ -55664,7 +55685,7 @@
         <v>8863</v>
       </c>
       <c r="B1086" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="C1086" t="s">
         <v>1163</v>
@@ -55682,7 +55703,7 @@
         <v>0</v>
       </c>
       <c r="H1086" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="I1086" t="s">
         <v>19</v>
@@ -55711,7 +55732,7 @@
         <v>8864</v>
       </c>
       <c r="B1087" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="C1087" t="s">
         <v>1163</v>
@@ -55729,7 +55750,7 @@
         <v>0</v>
       </c>
       <c r="H1087" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
       <c r="I1087" t="s">
         <v>19</v>
@@ -55758,7 +55779,7 @@
         <v>8865</v>
       </c>
       <c r="B1088" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="C1088" t="s">
         <v>1163</v>
@@ -55776,7 +55797,7 @@
         <v>0</v>
       </c>
       <c r="H1088" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
       <c r="I1088" t="s">
         <v>19</v>
@@ -55805,7 +55826,7 @@
         <v>8866</v>
       </c>
       <c r="B1089" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="C1089" t="s">
         <v>1163</v>
@@ -55852,7 +55873,7 @@
         <v>8867</v>
       </c>
       <c r="B1090" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="C1090" t="s">
         <v>1163</v>
@@ -55899,7 +55920,7 @@
         <v>8868</v>
       </c>
       <c r="B1091" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="C1091" t="s">
         <v>1163</v>
@@ -55946,7 +55967,7 @@
         <v>8869</v>
       </c>
       <c r="B1092" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
       <c r="C1092" t="s">
         <v>1163</v>
@@ -55993,7 +56014,7 @@
         <v>8870</v>
       </c>
       <c r="B1093" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="C1093" t="s">
         <v>1163</v>
@@ -56040,7 +56061,7 @@
         <v>8871</v>
       </c>
       <c r="B1094" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="C1094" t="s">
         <v>1163</v>
@@ -56087,7 +56108,7 @@
         <v>8872</v>
       </c>
       <c r="B1095" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
       <c r="C1095" t="s">
         <v>1163</v>
@@ -56134,7 +56155,7 @@
         <v>8873</v>
       </c>
       <c r="B1096" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="C1096" t="s">
         <v>1163</v>
@@ -56181,7 +56202,7 @@
         <v>8874</v>
       </c>
       <c r="B1097" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
       <c r="C1097" t="s">
         <v>1163</v>
@@ -56228,7 +56249,7 @@
         <v>8875</v>
       </c>
       <c r="B1098" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="C1098" t="s">
         <v>1163</v>
@@ -56275,7 +56296,7 @@
         <v>8876</v>
       </c>
       <c r="B1099" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
       <c r="C1099" t="s">
         <v>1163</v>
@@ -56322,7 +56343,7 @@
         <v>8877</v>
       </c>
       <c r="B1100" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="C1100" t="s">
         <v>1163</v>
@@ -56369,7 +56390,7 @@
         <v>8878</v>
       </c>
       <c r="B1101" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="C1101" t="s">
         <v>1163</v>
@@ -56416,7 +56437,7 @@
         <v>8879</v>
       </c>
       <c r="B1102" t="s">
-        <v>1208</v>
+        <v>1207</v>
       </c>
       <c r="C1102" t="s">
         <v>1163</v>
@@ -56463,7 +56484,7 @@
         <v>8880</v>
       </c>
       <c r="B1103" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
       <c r="C1103" t="s">
         <v>1163</v>
@@ -56510,7 +56531,7 @@
         <v>8881</v>
       </c>
       <c r="B1104" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="C1104" t="s">
         <v>1163</v>
@@ -56557,7 +56578,7 @@
         <v>8882</v>
       </c>
       <c r="B1105" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
       <c r="C1105" t="s">
         <v>1163</v>
@@ -56604,7 +56625,7 @@
         <v>8883</v>
       </c>
       <c r="B1106" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="C1106" t="s">
         <v>1163</v>
@@ -56651,7 +56672,7 @@
         <v>8884</v>
       </c>
       <c r="B1107" t="s">
-        <v>1213</v>
+        <v>1212</v>
       </c>
       <c r="C1107" t="s">
         <v>1163</v>
@@ -56698,7 +56719,7 @@
         <v>8885</v>
       </c>
       <c r="B1108" t="s">
-        <v>1214</v>
+        <v>1213</v>
       </c>
       <c r="C1108" t="s">
         <v>1163</v>
@@ -56745,7 +56766,7 @@
         <v>8886</v>
       </c>
       <c r="B1109" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="C1109" t="s">
         <v>1163</v>
@@ -56792,7 +56813,7 @@
         <v>8887</v>
       </c>
       <c r="B1110" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="C1110" t="s">
         <v>1163</v>
@@ -56839,7 +56860,7 @@
         <v>8888</v>
       </c>
       <c r="B1111" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
       <c r="C1111" t="s">
         <v>952</v>
@@ -56857,7 +56878,7 @@
         <v>0</v>
       </c>
       <c r="H1111" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="I1111" t="s">
         <v>19</v>
@@ -56886,7 +56907,7 @@
         <v>8889</v>
       </c>
       <c r="B1112" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
       <c r="C1112" t="s">
         <v>952</v>
@@ -56904,7 +56925,7 @@
         <v>0</v>
       </c>
       <c r="H1112" t="s">
-        <v>1219</v>
+        <v>1218</v>
       </c>
       <c r="I1112" t="s">
         <v>19</v>
@@ -56933,7 +56954,7 @@
         <v>8890</v>
       </c>
       <c r="B1113" t="s">
-        <v>1220</v>
+        <v>1219</v>
       </c>
       <c r="C1113" t="s">
         <v>952</v>
@@ -56951,7 +56972,7 @@
         <v>0</v>
       </c>
       <c r="H1113" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="I1113" t="s">
         <v>19</v>
@@ -56980,7 +57001,7 @@
         <v>8891</v>
       </c>
       <c r="B1114" t="s">
-        <v>1221</v>
+        <v>1220</v>
       </c>
       <c r="C1114" t="s">
         <v>952</v>
@@ -57027,7 +57048,7 @@
         <v>8892</v>
       </c>
       <c r="B1115" t="s">
-        <v>1222</v>
+        <v>1221</v>
       </c>
       <c r="C1115" t="s">
         <v>952</v>
@@ -57045,7 +57066,7 @@
         <v>0</v>
       </c>
       <c r="H1115" t="s">
-        <v>1223</v>
+        <v>1222</v>
       </c>
       <c r="I1115" t="s">
         <v>19</v>
@@ -57074,7 +57095,7 @@
         <v>8893</v>
       </c>
       <c r="B1116" t="s">
-        <v>1224</v>
+        <v>1223</v>
       </c>
       <c r="C1116" t="s">
         <v>952</v>
@@ -57121,7 +57142,7 @@
         <v>8894</v>
       </c>
       <c r="B1117" t="s">
-        <v>1225</v>
+        <v>1224</v>
       </c>
       <c r="C1117" t="s">
         <v>952</v>
@@ -57168,7 +57189,7 @@
         <v>8895</v>
       </c>
       <c r="B1118" t="s">
-        <v>1226</v>
+        <v>1225</v>
       </c>
       <c r="C1118" t="s">
         <v>952</v>
@@ -57215,7 +57236,7 @@
         <v>8896</v>
       </c>
       <c r="B1119" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C1119" t="s">
         <v>952</v>
@@ -57262,7 +57283,7 @@
         <v>8897</v>
       </c>
       <c r="B1120" t="s">
-        <v>1228</v>
+        <v>1227</v>
       </c>
       <c r="C1120" t="s">
         <v>952</v>
@@ -57309,7 +57330,7 @@
         <v>8898</v>
       </c>
       <c r="B1121" t="s">
-        <v>1229</v>
+        <v>1228</v>
       </c>
       <c r="C1121" t="s">
         <v>952</v>
@@ -57356,7 +57377,7 @@
         <v>8899</v>
       </c>
       <c r="B1122" t="s">
-        <v>1230</v>
+        <v>1229</v>
       </c>
       <c r="C1122" t="s">
         <v>952</v>
@@ -57403,7 +57424,7 @@
         <v>8900</v>
       </c>
       <c r="B1123" t="s">
-        <v>1231</v>
+        <v>1230</v>
       </c>
       <c r="C1123" t="s">
         <v>749</v>
@@ -57421,7 +57442,7 @@
         <v>0</v>
       </c>
       <c r="H1123" t="s">
-        <v>1232</v>
+        <v>1231</v>
       </c>
       <c r="I1123" t="s">
         <v>19</v>
@@ -57450,7 +57471,7 @@
         <v>8901</v>
       </c>
       <c r="B1124" t="s">
-        <v>1233</v>
+        <v>1232</v>
       </c>
       <c r="C1124" t="s">
         <v>749</v>
@@ -57468,7 +57489,7 @@
         <v>0</v>
       </c>
       <c r="H1124" t="s">
-        <v>1234</v>
+        <v>1233</v>
       </c>
       <c r="I1124" t="s">
         <v>19</v>
@@ -57497,7 +57518,7 @@
         <v>8902</v>
       </c>
       <c r="B1125" t="s">
-        <v>1235</v>
+        <v>1234</v>
       </c>
       <c r="C1125" t="s">
         <v>749</v>
@@ -57515,7 +57536,7 @@
         <v>0</v>
       </c>
       <c r="H1125" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="I1125" t="s">
         <v>19</v>
@@ -57544,7 +57565,7 @@
         <v>8903</v>
       </c>
       <c r="B1126" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
       <c r="C1126" t="s">
         <v>749</v>
@@ -57591,7 +57612,7 @@
         <v>8904</v>
       </c>
       <c r="B1127" t="s">
-        <v>1238</v>
+        <v>1237</v>
       </c>
       <c r="C1127" t="s">
         <v>749</v>
@@ -57638,7 +57659,7 @@
         <v>8905</v>
       </c>
       <c r="B1128" t="s">
-        <v>1239</v>
+        <v>1238</v>
       </c>
       <c r="C1128" t="s">
         <v>749</v>
@@ -57685,7 +57706,7 @@
         <v>8906</v>
       </c>
       <c r="B1129" t="s">
-        <v>1240</v>
+        <v>1239</v>
       </c>
       <c r="C1129" t="s">
         <v>749</v>
@@ -57732,7 +57753,7 @@
         <v>8907</v>
       </c>
       <c r="B1130" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
       <c r="C1130" t="s">
         <v>749</v>
@@ -57779,7 +57800,7 @@
         <v>8908</v>
       </c>
       <c r="B1131" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
       <c r="C1131" t="s">
         <v>749</v>
@@ -57826,7 +57847,7 @@
         <v>8909</v>
       </c>
       <c r="B1132" t="s">
-        <v>1243</v>
+        <v>1242</v>
       </c>
       <c r="C1132" t="s">
         <v>749</v>
@@ -57873,7 +57894,7 @@
         <v>8910</v>
       </c>
       <c r="B1133" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="C1133" t="s">
         <v>749</v>
@@ -57920,7 +57941,7 @@
         <v>8911</v>
       </c>
       <c r="B1134" t="s">
-        <v>1245</v>
+        <v>1244</v>
       </c>
       <c r="C1134" t="s">
         <v>749</v>
@@ -57967,7 +57988,7 @@
         <v>8912</v>
       </c>
       <c r="B1135" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="C1135" t="s">
         <v>749</v>
@@ -58014,7 +58035,7 @@
         <v>8913</v>
       </c>
       <c r="B1136" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="C1136" t="s">
         <v>749</v>
@@ -58061,7 +58082,7 @@
         <v>8914</v>
       </c>
       <c r="B1137" t="s">
-        <v>1248</v>
+        <v>1247</v>
       </c>
       <c r="C1137" t="s">
         <v>749</v>
@@ -58108,7 +58129,7 @@
         <v>8915</v>
       </c>
       <c r="B1138" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="C1138" t="s">
         <v>656</v>
@@ -58126,7 +58147,7 @@
         <v>0</v>
       </c>
       <c r="H1138" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="I1138" t="s">
         <v>19</v>
@@ -58155,7 +58176,7 @@
         <v>8916</v>
       </c>
       <c r="B1139" t="s">
-        <v>1250</v>
+        <v>1249</v>
       </c>
       <c r="C1139" t="s">
         <v>656</v>
@@ -58173,7 +58194,7 @@
         <v>0</v>
       </c>
       <c r="H1139" t="s">
-        <v>1232</v>
+        <v>1231</v>
       </c>
       <c r="I1139" t="s">
         <v>19</v>
@@ -58202,7 +58223,7 @@
         <v>8917</v>
       </c>
       <c r="B1140" t="s">
-        <v>1251</v>
+        <v>1250</v>
       </c>
       <c r="C1140" t="s">
         <v>656</v>
@@ -58249,7 +58270,7 @@
         <v>8918</v>
       </c>
       <c r="B1141" t="s">
-        <v>1252</v>
+        <v>1251</v>
       </c>
       <c r="C1141" t="s">
         <v>656</v>
@@ -58343,7 +58364,7 @@
         <v>8920</v>
       </c>
       <c r="B1143" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="C1143" t="s">
         <v>656</v>
@@ -58390,7 +58411,7 @@
         <v>8921</v>
       </c>
       <c r="B1144" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="C1144" t="s">
         <v>656</v>
@@ -58437,7 +58458,7 @@
         <v>8922</v>
       </c>
       <c r="B1145" t="s">
-        <v>1255</v>
+        <v>1254</v>
       </c>
       <c r="C1145" t="s">
         <v>656</v>
@@ -58484,7 +58505,7 @@
         <v>8923</v>
       </c>
       <c r="B1146" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
       <c r="C1146" t="s">
         <v>656</v>
@@ -58531,7 +58552,7 @@
         <v>8924</v>
       </c>
       <c r="B1147" t="s">
-        <v>1257</v>
+        <v>1256</v>
       </c>
       <c r="C1147" t="s">
         <v>656</v>
@@ -58578,7 +58599,7 @@
         <v>8925</v>
       </c>
       <c r="B1148" t="s">
-        <v>1258</v>
+        <v>1257</v>
       </c>
       <c r="C1148" t="s">
         <v>656</v>
@@ -58625,7 +58646,7 @@
         <v>8926</v>
       </c>
       <c r="B1149" t="s">
-        <v>1259</v>
+        <v>1258</v>
       </c>
       <c r="C1149" t="s">
         <v>656</v>
@@ -58672,7 +58693,7 @@
         <v>8927</v>
       </c>
       <c r="B1150" t="s">
-        <v>1260</v>
+        <v>1259</v>
       </c>
       <c r="C1150" t="s">
         <v>656</v>
@@ -58719,7 +58740,7 @@
         <v>8928</v>
       </c>
       <c r="B1151" t="s">
-        <v>1261</v>
+        <v>1260</v>
       </c>
       <c r="C1151" t="s">
         <v>537</v>
@@ -58737,7 +58758,7 @@
         <v>7690</v>
       </c>
       <c r="H1151" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
       <c r="I1151" t="s">
         <v>19</v>
@@ -58766,7 +58787,7 @@
         <v>8929</v>
       </c>
       <c r="B1152" t="s">
-        <v>1263</v>
+        <v>1262</v>
       </c>
       <c r="C1152" t="s">
         <v>537</v>
@@ -58784,7 +58805,7 @@
         <v>0</v>
       </c>
       <c r="H1152" t="s">
-        <v>1219</v>
+        <v>1218</v>
       </c>
       <c r="I1152" t="s">
         <v>19</v>
@@ -58813,7 +58834,7 @@
         <v>8930</v>
       </c>
       <c r="B1153" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
       <c r="C1153" t="s">
         <v>537</v>
@@ -58831,7 +58852,7 @@
         <v>0</v>
       </c>
       <c r="H1153" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="I1153" t="s">
         <v>19</v>
@@ -58860,7 +58881,7 @@
         <v>8931</v>
       </c>
       <c r="B1154" t="s">
-        <v>1265</v>
+        <v>1264</v>
       </c>
       <c r="C1154" t="s">
         <v>537</v>
@@ -58878,7 +58899,7 @@
         <v>0</v>
       </c>
       <c r="H1154" t="s">
-        <v>1223</v>
+        <v>1222</v>
       </c>
       <c r="I1154" t="s">
         <v>19</v>
@@ -58907,7 +58928,7 @@
         <v>8932</v>
       </c>
       <c r="B1155" t="s">
-        <v>1266</v>
+        <v>1265</v>
       </c>
       <c r="C1155" t="s">
         <v>537</v>
@@ -58954,7 +58975,7 @@
         <v>8933</v>
       </c>
       <c r="B1156" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="C1156" t="s">
         <v>537</v>
@@ -59001,7 +59022,7 @@
         <v>8934</v>
       </c>
       <c r="B1157" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="C1157" t="s">
         <v>537</v>
@@ -59048,7 +59069,7 @@
         <v>8935</v>
       </c>
       <c r="B1158" t="s">
-        <v>1269</v>
+        <v>1268</v>
       </c>
       <c r="C1158" t="s">
         <v>537</v>
@@ -59095,7 +59116,7 @@
         <v>8936</v>
       </c>
       <c r="B1159" t="s">
-        <v>1270</v>
+        <v>1269</v>
       </c>
       <c r="C1159" t="s">
         <v>537</v>
@@ -59142,7 +59163,7 @@
         <v>8937</v>
       </c>
       <c r="B1160" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="C1160" t="s">
         <v>537</v>
@@ -59189,7 +59210,7 @@
         <v>8938</v>
       </c>
       <c r="B1161" t="s">
-        <v>1272</v>
+        <v>1271</v>
       </c>
       <c r="C1161" t="s">
         <v>537</v>
@@ -59236,7 +59257,7 @@
         <v>8939</v>
       </c>
       <c r="B1162" t="s">
-        <v>1273</v>
+        <v>1272</v>
       </c>
       <c r="C1162" t="s">
         <v>537</v>
@@ -59283,7 +59304,7 @@
         <v>8940</v>
       </c>
       <c r="B1163" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
       <c r="C1163" t="s">
         <v>537</v>
@@ -59330,7 +59351,7 @@
         <v>8941</v>
       </c>
       <c r="B1164" t="s">
-        <v>1275</v>
+        <v>1274</v>
       </c>
       <c r="C1164" t="s">
         <v>537</v>
@@ -59377,7 +59398,7 @@
         <v>8942</v>
       </c>
       <c r="B1165" t="s">
-        <v>1276</v>
+        <v>1275</v>
       </c>
       <c r="C1165" t="s">
         <v>550</v>
@@ -59424,7 +59445,7 @@
         <v>8943</v>
       </c>
       <c r="B1166" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
       <c r="C1166" t="s">
         <v>550</v>
@@ -59442,7 +59463,7 @@
         <v>0</v>
       </c>
       <c r="H1166" t="s">
-        <v>1278</v>
+        <v>1277</v>
       </c>
       <c r="I1166" t="s">
         <v>19</v>
@@ -59471,7 +59492,7 @@
         <v>8944</v>
       </c>
       <c r="B1167" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
       <c r="C1167" t="s">
         <v>550</v>
@@ -59518,7 +59539,7 @@
         <v>8945</v>
       </c>
       <c r="B1168" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
       <c r="C1168" t="s">
         <v>550</v>
@@ -59565,7 +59586,7 @@
         <v>8946</v>
       </c>
       <c r="B1169" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
       <c r="C1169" t="s">
         <v>550</v>
@@ -59612,7 +59633,7 @@
         <v>8947</v>
       </c>
       <c r="B1170" t="s">
-        <v>1282</v>
+        <v>1281</v>
       </c>
       <c r="C1170" t="s">
         <v>550</v>
@@ -59659,7 +59680,7 @@
         <v>8948</v>
       </c>
       <c r="B1171" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
       <c r="C1171" t="s">
         <v>550</v>
@@ -59706,7 +59727,7 @@
         <v>8949</v>
       </c>
       <c r="B1172" t="s">
-        <v>1284</v>
+        <v>1283</v>
       </c>
       <c r="C1172" t="s">
         <v>550</v>
@@ -59753,7 +59774,7 @@
         <v>8950</v>
       </c>
       <c r="B1173" t="s">
-        <v>1285</v>
+        <v>1284</v>
       </c>
       <c r="C1173" t="s">
         <v>550</v>
@@ -59800,7 +59821,7 @@
         <v>8951</v>
       </c>
       <c r="B1174" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
       <c r="C1174" t="s">
         <v>497</v>
@@ -59818,7 +59839,7 @@
         <v>0</v>
       </c>
       <c r="H1174" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="I1174" t="s">
         <v>19</v>
@@ -59847,7 +59868,7 @@
         <v>8952</v>
       </c>
       <c r="B1175" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
       <c r="C1175" t="s">
         <v>497</v>
@@ -59894,7 +59915,7 @@
         <v>8953</v>
       </c>
       <c r="B1176" t="s">
-        <v>1288</v>
+        <v>1287</v>
       </c>
       <c r="C1176" t="s">
         <v>497</v>
@@ -59941,7 +59962,7 @@
         <v>8954</v>
       </c>
       <c r="B1177" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
       <c r="C1177" t="s">
         <v>497</v>
@@ -59988,7 +60009,7 @@
         <v>8955</v>
       </c>
       <c r="B1178" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
       <c r="C1178" t="s">
         <v>497</v>
@@ -60035,7 +60056,7 @@
         <v>8956</v>
       </c>
       <c r="B1179" t="s">
-        <v>1291</v>
+        <v>1290</v>
       </c>
       <c r="C1179" t="s">
         <v>497</v>
@@ -60082,7 +60103,7 @@
         <v>8957</v>
       </c>
       <c r="B1180" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
       <c r="C1180" t="s">
         <v>497</v>
@@ -60129,7 +60150,7 @@
         <v>8958</v>
       </c>
       <c r="B1181" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="C1181" t="s">
         <v>497</v>
@@ -60176,7 +60197,7 @@
         <v>8959</v>
       </c>
       <c r="B1182" t="s">
-        <v>1294</v>
+        <v>1293</v>
       </c>
       <c r="C1182" t="s">
         <v>497</v>
@@ -60223,7 +60244,7 @@
         <v>8960</v>
       </c>
       <c r="B1183" t="s">
-        <v>1295</v>
+        <v>1294</v>
       </c>
       <c r="C1183" t="s">
         <v>497</v>
@@ -60270,7 +60291,7 @@
         <v>8961</v>
       </c>
       <c r="B1184" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
       <c r="C1184" t="s">
         <v>497</v>
@@ -60317,7 +60338,7 @@
         <v>8962</v>
       </c>
       <c r="B1185" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
       <c r="C1185" t="s">
         <v>497</v>
@@ -60364,7 +60385,7 @@
         <v>8963</v>
       </c>
       <c r="B1186" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
       <c r="C1186" t="s">
         <v>497</v>
@@ -60411,7 +60432,7 @@
         <v>8964</v>
       </c>
       <c r="B1187" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="C1187" t="s">
         <v>497</v>
@@ -60458,7 +60479,7 @@
         <v>8965</v>
       </c>
       <c r="B1188" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="C1188" t="s">
         <v>464</v>
@@ -60505,7 +60526,7 @@
         <v>8966</v>
       </c>
       <c r="B1189" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="C1189" t="s">
         <v>464</v>
@@ -60523,7 +60544,7 @@
         <v>0</v>
       </c>
       <c r="H1189" t="s">
-        <v>1278</v>
+        <v>1277</v>
       </c>
       <c r="I1189" t="s">
         <v>19</v>
@@ -60552,7 +60573,7 @@
         <v>8967</v>
       </c>
       <c r="B1190" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
       <c r="C1190" t="s">
         <v>464</v>
@@ -60599,7 +60620,7 @@
         <v>8968</v>
       </c>
       <c r="B1191" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
       <c r="C1191" t="s">
         <v>464</v>
@@ -60646,7 +60667,7 @@
         <v>8969</v>
       </c>
       <c r="B1192" t="s">
-        <v>1304</v>
+        <v>1303</v>
       </c>
       <c r="C1192" t="s">
         <v>464</v>
@@ -60693,7 +60714,7 @@
         <v>8970</v>
       </c>
       <c r="B1193" t="s">
-        <v>1305</v>
+        <v>1304</v>
       </c>
       <c r="C1193" t="s">
         <v>464</v>
@@ -60740,7 +60761,7 @@
         <v>8971</v>
       </c>
       <c r="B1194" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="C1194" t="s">
         <v>464</v>
@@ -60787,7 +60808,7 @@
         <v>8972</v>
       </c>
       <c r="B1195" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="C1195" t="s">
         <v>464</v>
@@ -60834,7 +60855,7 @@
         <v>8973</v>
       </c>
       <c r="B1196" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
       <c r="C1196" t="s">
         <v>464</v>
@@ -60881,7 +60902,7 @@
         <v>8974</v>
       </c>
       <c r="B1197" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
       <c r="C1197" t="s">
         <v>464</v>
@@ -60928,7 +60949,7 @@
         <v>8975</v>
       </c>
       <c r="B1198" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
       <c r="C1198" t="s">
         <v>464</v>
@@ -60975,7 +60996,7 @@
         <v>8976</v>
       </c>
       <c r="B1199" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="C1199" t="s">
         <v>464</v>
@@ -61022,7 +61043,7 @@
         <v>8977</v>
       </c>
       <c r="B1200" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="C1200" t="s">
         <v>464</v>
@@ -61069,7 +61090,7 @@
         <v>8978</v>
       </c>
       <c r="B1201" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
       <c r="C1201" t="s">
         <v>464</v>
@@ -61116,7 +61137,7 @@
         <v>8979</v>
       </c>
       <c r="B1202" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
       <c r="C1202" t="s">
         <v>464</v>
@@ -61163,7 +61184,7 @@
         <v>8980</v>
       </c>
       <c r="B1203" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="C1203" t="s">
         <v>464</v>
@@ -61210,7 +61231,7 @@
         <v>8981</v>
       </c>
       <c r="B1204" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
       <c r="C1204" t="s">
         <v>464</v>
@@ -61257,7 +61278,7 @@
         <v>8982</v>
       </c>
       <c r="B1205" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
       <c r="C1205" t="s">
         <v>464</v>
@@ -61304,7 +61325,7 @@
         <v>8983</v>
       </c>
       <c r="B1206" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
       <c r="C1206" t="s">
         <v>464</v>
@@ -61351,7 +61372,7 @@
         <v>8984</v>
       </c>
       <c r="B1207" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
       <c r="C1207" t="s">
         <v>464</v>
@@ -61398,7 +61419,7 @@
         <v>8985</v>
       </c>
       <c r="B1208" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
       <c r="C1208" t="s">
         <v>464</v>
@@ -61445,7 +61466,7 @@
         <v>8986</v>
       </c>
       <c r="B1209" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="C1209" t="s">
         <v>464</v>
@@ -61492,7 +61513,7 @@
         <v>8987</v>
       </c>
       <c r="B1210" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
       <c r="C1210" t="s">
         <v>464</v>
@@ -61539,7 +61560,7 @@
         <v>8988</v>
       </c>
       <c r="B1211" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
       <c r="C1211" t="s">
         <v>464</v>
@@ -61586,7 +61607,7 @@
         <v>8989</v>
       </c>
       <c r="B1212" t="s">
-        <v>1324</v>
+        <v>1323</v>
       </c>
       <c r="C1212" t="s">
         <v>464</v>
@@ -61633,7 +61654,7 @@
         <v>8990</v>
       </c>
       <c r="B1213" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
       <c r="C1213" t="s">
         <v>464</v>
@@ -61680,7 +61701,7 @@
         <v>8991</v>
       </c>
       <c r="B1214" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
       <c r="C1214" t="s">
         <v>464</v>
@@ -61727,7 +61748,7 @@
         <v>8992</v>
       </c>
       <c r="B1215" t="s">
-        <v>1327</v>
+        <v>1326</v>
       </c>
       <c r="C1215" t="s">
         <v>464</v>
@@ -61774,7 +61795,7 @@
         <v>8993</v>
       </c>
       <c r="B1216" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
       <c r="C1216" t="s">
         <v>464</v>
@@ -61821,7 +61842,7 @@
         <v>8994</v>
       </c>
       <c r="B1217" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="C1217" t="s">
         <v>464</v>
@@ -61868,7 +61889,7 @@
         <v>8995</v>
       </c>
       <c r="B1218" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="C1218" t="s">
         <v>464</v>
@@ -61915,7 +61936,7 @@
         <v>8996</v>
       </c>
       <c r="B1219" t="s">
-        <v>1331</v>
+        <v>1330</v>
       </c>
       <c r="C1219" t="s">
         <v>464</v>
@@ -61962,7 +61983,7 @@
         <v>8997</v>
       </c>
       <c r="B1220" t="s">
-        <v>1332</v>
+        <v>1331</v>
       </c>
       <c r="C1220" t="s">
         <v>464</v>
@@ -62009,7 +62030,7 @@
         <v>8998</v>
       </c>
       <c r="B1221" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="C1221" t="s">
         <v>464</v>
@@ -62056,7 +62077,7 @@
         <v>8999</v>
       </c>
       <c r="B1222" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="C1222" t="s">
         <v>464</v>
@@ -62103,7 +62124,7 @@
         <v>9000</v>
       </c>
       <c r="B1223" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="C1223" t="s">
         <v>464</v>
@@ -62150,7 +62171,7 @@
         <v>9001</v>
       </c>
       <c r="B1224" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="C1224" t="s">
         <v>464</v>
@@ -62244,7 +62265,7 @@
         <v>9003</v>
       </c>
       <c r="B1226" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="C1226" t="s">
         <v>427</v>
@@ -62262,7 +62283,7 @@
         <v>0</v>
       </c>
       <c r="H1226" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="I1226" t="s">
         <v>19</v>
@@ -62291,7 +62312,7 @@
         <v>9004</v>
       </c>
       <c r="B1227" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="C1227" t="s">
         <v>427</v>
@@ -62338,7 +62359,7 @@
         <v>9005</v>
       </c>
       <c r="B1228" t="s">
-        <v>1340</v>
+        <v>1339</v>
       </c>
       <c r="C1228" t="s">
         <v>427</v>
@@ -62385,7 +62406,7 @@
         <v>9006</v>
       </c>
       <c r="B1229" t="s">
-        <v>1341</v>
+        <v>1340</v>
       </c>
       <c r="C1229" t="s">
         <v>427</v>
@@ -62432,7 +62453,7 @@
         <v>9007</v>
       </c>
       <c r="B1230" t="s">
-        <v>1342</v>
+        <v>1341</v>
       </c>
       <c r="C1230" t="s">
         <v>427</v>
@@ -62479,7 +62500,7 @@
         <v>9008</v>
       </c>
       <c r="B1231" t="s">
-        <v>1343</v>
+        <v>1342</v>
       </c>
       <c r="C1231" t="s">
         <v>427</v>
@@ -62526,7 +62547,7 @@
         <v>9009</v>
       </c>
       <c r="B1232" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="C1232" t="s">
         <v>427</v>
@@ -62573,7 +62594,7 @@
         <v>9010</v>
       </c>
       <c r="B1233" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="C1233" t="s">
         <v>427</v>
@@ -62620,7 +62641,7 @@
         <v>9011</v>
       </c>
       <c r="B1234" t="s">
-        <v>1346</v>
+        <v>1345</v>
       </c>
       <c r="C1234" t="s">
         <v>427</v>
@@ -62667,7 +62688,7 @@
         <v>9012</v>
       </c>
       <c r="B1235" t="s">
-        <v>1347</v>
+        <v>1346</v>
       </c>
       <c r="C1235" t="s">
         <v>427</v>
@@ -62714,7 +62735,7 @@
         <v>9013</v>
       </c>
       <c r="B1236" t="s">
-        <v>1348</v>
+        <v>1347</v>
       </c>
       <c r="C1236" t="s">
         <v>427</v>
@@ -62761,7 +62782,7 @@
         <v>9014</v>
       </c>
       <c r="B1237" t="s">
-        <v>1349</v>
+        <v>1348</v>
       </c>
       <c r="C1237" t="s">
         <v>427</v>
@@ -62808,7 +62829,7 @@
         <v>9015</v>
       </c>
       <c r="B1238" t="s">
-        <v>1350</v>
+        <v>1349</v>
       </c>
       <c r="C1238" t="s">
         <v>427</v>
@@ -62855,7 +62876,7 @@
         <v>9016</v>
       </c>
       <c r="B1239" t="s">
-        <v>1351</v>
+        <v>1350</v>
       </c>
       <c r="C1239" t="s">
         <v>427</v>
@@ -62902,7 +62923,7 @@
         <v>9017</v>
       </c>
       <c r="B1240" t="s">
-        <v>1352</v>
+        <v>1351</v>
       </c>
       <c r="C1240" t="s">
         <v>427</v>
@@ -62949,7 +62970,7 @@
         <v>9018</v>
       </c>
       <c r="B1241" t="s">
-        <v>1353</v>
+        <v>1352</v>
       </c>
       <c r="C1241" t="s">
         <v>427</v>
@@ -62996,7 +63017,7 @@
         <v>9019</v>
       </c>
       <c r="B1242" t="s">
-        <v>1354</v>
+        <v>1353</v>
       </c>
       <c r="C1242" t="s">
         <v>427</v>
@@ -63043,7 +63064,7 @@
         <v>9020</v>
       </c>
       <c r="B1243" t="s">
-        <v>1355</v>
+        <v>1354</v>
       </c>
       <c r="C1243" t="s">
         <v>427</v>
@@ -63090,7 +63111,7 @@
         <v>9021</v>
       </c>
       <c r="B1244" t="s">
-        <v>1356</v>
+        <v>1355</v>
       </c>
       <c r="C1244" t="s">
         <v>427</v>
@@ -63137,7 +63158,7 @@
         <v>9022</v>
       </c>
       <c r="B1245" t="s">
-        <v>1357</v>
+        <v>1356</v>
       </c>
       <c r="C1245" t="s">
         <v>427</v>
@@ -63184,7 +63205,7 @@
         <v>9023</v>
       </c>
       <c r="B1246" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="C1246" t="s">
         <v>427</v>
@@ -63231,7 +63252,7 @@
         <v>9024</v>
       </c>
       <c r="B1247" t="s">
-        <v>1359</v>
+        <v>1358</v>
       </c>
       <c r="C1247" t="s">
         <v>393</v>
@@ -63249,7 +63270,7 @@
         <v>0</v>
       </c>
       <c r="H1247" t="s">
-        <v>1223</v>
+        <v>1222</v>
       </c>
       <c r="I1247" t="s">
         <v>19</v>
@@ -63278,7 +63299,7 @@
         <v>9025</v>
       </c>
       <c r="B1248" t="s">
-        <v>1360</v>
+        <v>1359</v>
       </c>
       <c r="C1248" t="s">
         <v>393</v>
@@ -63296,7 +63317,7 @@
         <v>0</v>
       </c>
       <c r="H1248" t="s">
-        <v>1223</v>
+        <v>1222</v>
       </c>
       <c r="I1248" t="s">
         <v>19</v>
@@ -63325,7 +63346,7 @@
         <v>9026</v>
       </c>
       <c r="B1249" t="s">
-        <v>1361</v>
+        <v>1360</v>
       </c>
       <c r="C1249" t="s">
         <v>393</v>
@@ -63372,7 +63393,7 @@
         <v>9027</v>
       </c>
       <c r="B1250" t="s">
-        <v>1362</v>
+        <v>1361</v>
       </c>
       <c r="C1250" t="s">
         <v>393</v>
@@ -63419,7 +63440,7 @@
         <v>9028</v>
       </c>
       <c r="B1251" t="s">
-        <v>1363</v>
+        <v>1362</v>
       </c>
       <c r="C1251" t="s">
         <v>393</v>
@@ -63466,7 +63487,7 @@
         <v>9029</v>
       </c>
       <c r="B1252" t="s">
-        <v>1364</v>
+        <v>1363</v>
       </c>
       <c r="C1252" t="s">
         <v>393</v>
@@ -63513,7 +63534,7 @@
         <v>9030</v>
       </c>
       <c r="B1253" t="s">
-        <v>1365</v>
+        <v>1364</v>
       </c>
       <c r="C1253" t="s">
         <v>393</v>
@@ -63560,7 +63581,7 @@
         <v>9031</v>
       </c>
       <c r="B1254" t="s">
-        <v>1366</v>
+        <v>1365</v>
       </c>
       <c r="C1254" t="s">
         <v>393</v>
@@ -63607,7 +63628,7 @@
         <v>9032</v>
       </c>
       <c r="B1255" t="s">
-        <v>1367</v>
+        <v>1366</v>
       </c>
       <c r="C1255" t="s">
         <v>393</v>
@@ -63654,7 +63675,7 @@
         <v>9033</v>
       </c>
       <c r="B1256" t="s">
-        <v>1368</v>
+        <v>1367</v>
       </c>
       <c r="C1256" t="s">
         <v>393</v>
@@ -63701,7 +63722,7 @@
         <v>9034</v>
       </c>
       <c r="B1257" t="s">
-        <v>1369</v>
+        <v>1368</v>
       </c>
       <c r="C1257" t="s">
         <v>393</v>
@@ -63748,7 +63769,7 @@
         <v>9035</v>
       </c>
       <c r="B1258" t="s">
-        <v>1370</v>
+        <v>1369</v>
       </c>
       <c r="C1258" t="s">
         <v>393</v>
@@ -63795,7 +63816,7 @@
         <v>9036</v>
       </c>
       <c r="B1259" t="s">
-        <v>1371</v>
+        <v>1370</v>
       </c>
       <c r="C1259" t="s">
         <v>393</v>
@@ -63842,7 +63863,7 @@
         <v>9037</v>
       </c>
       <c r="B1260" t="s">
-        <v>1372</v>
+        <v>1371</v>
       </c>
       <c r="C1260" t="s">
         <v>393</v>
@@ -63889,7 +63910,7 @@
         <v>9038</v>
       </c>
       <c r="B1261" t="s">
-        <v>1373</v>
+        <v>1372</v>
       </c>
       <c r="C1261" t="s">
         <v>393</v>
@@ -63936,7 +63957,7 @@
         <v>9039</v>
       </c>
       <c r="B1262" t="s">
-        <v>1374</v>
+        <v>1373</v>
       </c>
       <c r="C1262" t="s">
         <v>427</v>
@@ -63983,7 +64004,7 @@
         <v>9040</v>
       </c>
       <c r="B1263" t="s">
-        <v>1375</v>
+        <v>1374</v>
       </c>
       <c r="C1263" t="s">
         <v>393</v>
@@ -64030,7 +64051,7 @@
         <v>9041</v>
       </c>
       <c r="B1264" t="s">
-        <v>1376</v>
+        <v>1375</v>
       </c>
       <c r="C1264" t="s">
         <v>393</v>
@@ -64077,7 +64098,7 @@
         <v>9042</v>
       </c>
       <c r="B1265" t="s">
-        <v>1377</v>
+        <v>1376</v>
       </c>
       <c r="C1265" t="s">
         <v>393</v>
@@ -64124,7 +64145,7 @@
         <v>9043</v>
       </c>
       <c r="B1266" t="s">
-        <v>1378</v>
+        <v>1377</v>
       </c>
       <c r="C1266" t="s">
         <v>393</v>
@@ -64171,7 +64192,7 @@
         <v>9044</v>
       </c>
       <c r="B1267" t="s">
-        <v>1379</v>
+        <v>1378</v>
       </c>
       <c r="C1267" t="s">
         <v>393</v>
@@ -64218,7 +64239,7 @@
         <v>9045</v>
       </c>
       <c r="B1268" t="s">
-        <v>1380</v>
+        <v>1379</v>
       </c>
       <c r="C1268" t="s">
         <v>393</v>
@@ -64265,7 +64286,7 @@
         <v>9046</v>
       </c>
       <c r="B1269" t="s">
-        <v>1381</v>
+        <v>1380</v>
       </c>
       <c r="C1269" t="s">
         <v>393</v>
@@ -64312,7 +64333,7 @@
         <v>9047</v>
       </c>
       <c r="B1270" t="s">
-        <v>1382</v>
+        <v>1381</v>
       </c>
       <c r="C1270" t="s">
         <v>393</v>
@@ -64359,7 +64380,7 @@
         <v>9048</v>
       </c>
       <c r="B1271" t="s">
-        <v>1383</v>
+        <v>1382</v>
       </c>
       <c r="C1271" t="s">
         <v>393</v>
@@ -64406,7 +64427,7 @@
         <v>9049</v>
       </c>
       <c r="B1272" t="s">
-        <v>1384</v>
+        <v>1383</v>
       </c>
       <c r="C1272" t="s">
         <v>393</v>
@@ -64453,7 +64474,7 @@
         <v>9050</v>
       </c>
       <c r="B1273" t="s">
-        <v>1235</v>
+        <v>1234</v>
       </c>
       <c r="C1273" t="s">
         <v>393</v>
@@ -64500,7 +64521,7 @@
         <v>9051</v>
       </c>
       <c r="B1274" t="s">
-        <v>1385</v>
+        <v>1384</v>
       </c>
       <c r="C1274" t="s">
         <v>342</v>
@@ -64518,7 +64539,7 @@
         <v>0</v>
       </c>
       <c r="H1274" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="I1274" t="s">
         <v>19</v>
@@ -64547,7 +64568,7 @@
         <v>9052</v>
       </c>
       <c r="B1275" t="s">
-        <v>1386</v>
+        <v>1385</v>
       </c>
       <c r="C1275" t="s">
         <v>342</v>
@@ -64565,7 +64586,7 @@
         <v>0</v>
       </c>
       <c r="H1275" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="I1275" t="s">
         <v>19</v>
@@ -64594,7 +64615,7 @@
         <v>9053</v>
       </c>
       <c r="B1276" t="s">
-        <v>1387</v>
+        <v>1386</v>
       </c>
       <c r="C1276" t="s">
         <v>342</v>
@@ -64641,7 +64662,7 @@
         <v>9054</v>
       </c>
       <c r="B1277" t="s">
-        <v>1388</v>
+        <v>1387</v>
       </c>
       <c r="C1277" t="s">
         <v>342</v>
@@ -64688,7 +64709,7 @@
         <v>9055</v>
       </c>
       <c r="B1278" t="s">
-        <v>1389</v>
+        <v>1388</v>
       </c>
       <c r="C1278" t="s">
         <v>342</v>
@@ -64735,7 +64756,7 @@
         <v>9056</v>
       </c>
       <c r="B1279" t="s">
-        <v>1390</v>
+        <v>1389</v>
       </c>
       <c r="C1279" t="s">
         <v>342</v>
@@ -64782,7 +64803,7 @@
         <v>9057</v>
       </c>
       <c r="B1280" t="s">
-        <v>1391</v>
+        <v>1390</v>
       </c>
       <c r="C1280" t="s">
         <v>342</v>
@@ -64829,7 +64850,7 @@
         <v>9058</v>
       </c>
       <c r="B1281" t="s">
-        <v>1392</v>
+        <v>1391</v>
       </c>
       <c r="C1281" t="s">
         <v>342</v>
@@ -64876,7 +64897,7 @@
         <v>9060</v>
       </c>
       <c r="B1282" t="s">
-        <v>1393</v>
+        <v>1392</v>
       </c>
       <c r="C1282" t="s">
         <v>342</v>
@@ -64923,7 +64944,7 @@
         <v>9061</v>
       </c>
       <c r="B1283" t="s">
-        <v>1394</v>
+        <v>1393</v>
       </c>
       <c r="C1283" t="s">
         <v>342</v>
@@ -64970,7 +64991,7 @@
         <v>9062</v>
       </c>
       <c r="B1284" t="s">
-        <v>1395</v>
+        <v>1394</v>
       </c>
       <c r="C1284" t="s">
         <v>342</v>
@@ -65017,7 +65038,7 @@
         <v>9063</v>
       </c>
       <c r="B1285" t="s">
-        <v>1396</v>
+        <v>1395</v>
       </c>
       <c r="C1285" t="s">
         <v>342</v>
@@ -65064,7 +65085,7 @@
         <v>9064</v>
       </c>
       <c r="B1286" t="s">
-        <v>1397</v>
+        <v>1396</v>
       </c>
       <c r="C1286" t="s">
         <v>342</v>
@@ -65158,7 +65179,7 @@
         <v>9066</v>
       </c>
       <c r="B1288" t="s">
-        <v>1398</v>
+        <v>1397</v>
       </c>
       <c r="C1288" t="s">
         <v>464</v>
@@ -65205,7 +65226,7 @@
         <v>9067</v>
       </c>
       <c r="B1289" t="s">
-        <v>1399</v>
+        <v>1398</v>
       </c>
       <c r="C1289" t="s">
         <v>1163</v>
@@ -65252,7 +65273,7 @@
         <v>9068</v>
       </c>
       <c r="B1290" t="s">
-        <v>1400</v>
+        <v>1399</v>
       </c>
       <c r="C1290" t="s">
         <v>952</v>
@@ -65270,7 +65291,7 @@
         <v>0</v>
       </c>
       <c r="H1290" t="s">
-        <v>1401</v>
+        <v>1400</v>
       </c>
       <c r="I1290" t="s">
         <v>19</v>
@@ -65299,7 +65320,7 @@
         <v>9069</v>
       </c>
       <c r="B1291" t="s">
-        <v>1402</v>
+        <v>1401</v>
       </c>
       <c r="C1291" t="s">
         <v>464</v>
@@ -65346,7 +65367,7 @@
         <v>9070</v>
       </c>
       <c r="B1292" t="s">
-        <v>1403</v>
+        <v>1402</v>
       </c>
       <c r="C1292" t="s">
         <v>550</v>
@@ -65393,7 +65414,7 @@
         <v>9071</v>
       </c>
       <c r="B1293" t="s">
-        <v>1404</v>
+        <v>1403</v>
       </c>
       <c r="C1293" t="s">
         <v>497</v>
@@ -65411,7 +65432,7 @@
         <v>0</v>
       </c>
       <c r="H1293" t="s">
-        <v>1405</v>
+        <v>1404</v>
       </c>
       <c r="I1293" t="s">
         <v>19</v>
@@ -65458,7 +65479,7 @@
         <v>0</v>
       </c>
       <c r="H1294" t="s">
-        <v>1405</v>
+        <v>1404</v>
       </c>
       <c r="I1294" t="s">
         <v>19</v>
@@ -65487,7 +65508,7 @@
         <v>9073</v>
       </c>
       <c r="B1295" t="s">
-        <v>1406</v>
+        <v>1405</v>
       </c>
       <c r="C1295" t="s">
         <v>1163</v>
@@ -65505,7 +65526,7 @@
         <v>0</v>
       </c>
       <c r="H1295" t="s">
-        <v>1405</v>
+        <v>1404</v>
       </c>
       <c r="I1295" t="s">
         <v>19</v>
@@ -65534,7 +65555,7 @@
         <v>9074</v>
       </c>
       <c r="B1296" t="s">
-        <v>1407</v>
+        <v>1406</v>
       </c>
       <c r="C1296" t="s">
         <v>1163</v>
@@ -65552,7 +65573,7 @@
         <v>0</v>
       </c>
       <c r="H1296" t="s">
-        <v>1405</v>
+        <v>1404</v>
       </c>
       <c r="I1296" t="s">
         <v>19</v>
@@ -65581,7 +65602,7 @@
         <v>9075</v>
       </c>
       <c r="B1297" t="s">
-        <v>1408</v>
+        <v>1407</v>
       </c>
       <c r="C1297" t="s">
         <v>952</v>
@@ -65628,7 +65649,7 @@
         <v>9076</v>
       </c>
       <c r="B1298" t="s">
-        <v>1409</v>
+        <v>1408</v>
       </c>
       <c r="C1298" t="s">
         <v>537</v>
@@ -65675,7 +65696,7 @@
         <v>9077</v>
       </c>
       <c r="B1299" t="s">
-        <v>1410</v>
+        <v>1409</v>
       </c>
       <c r="C1299" t="s">
         <v>497</v>
@@ -65722,7 +65743,7 @@
         <v>9078</v>
       </c>
       <c r="B1300" t="s">
-        <v>1411</v>
+        <v>1410</v>
       </c>
       <c r="C1300" t="s">
         <v>749</v>
@@ -65769,7 +65790,7 @@
         <v>9079</v>
       </c>
       <c r="B1301" t="s">
-        <v>1412</v>
+        <v>1411</v>
       </c>
       <c r="C1301" t="s">
         <v>342</v>
@@ -65787,7 +65808,7 @@
         <v>0</v>
       </c>
       <c r="H1301" t="s">
-        <v>1413</v>
+        <v>1412</v>
       </c>
       <c r="I1301" t="s">
         <v>19</v>
@@ -65816,7 +65837,7 @@
         <v>9080</v>
       </c>
       <c r="B1302" t="s">
-        <v>1414</v>
+        <v>1413</v>
       </c>
       <c r="C1302" t="s">
         <v>749</v>
@@ -65863,7 +65884,7 @@
         <v>9081</v>
       </c>
       <c r="B1303" t="s">
-        <v>1415</v>
+        <v>1414</v>
       </c>
       <c r="C1303" t="s">
         <v>393</v>
@@ -65881,7 +65902,7 @@
         <v>0</v>
       </c>
       <c r="H1303" t="s">
-        <v>1401</v>
+        <v>1400</v>
       </c>
       <c r="I1303" t="s">
         <v>19</v>
@@ -65910,7 +65931,7 @@
         <v>9082</v>
       </c>
       <c r="B1304" t="s">
-        <v>1416</v>
+        <v>1415</v>
       </c>
       <c r="C1304" t="s">
         <v>342</v>
@@ -65928,7 +65949,7 @@
         <v>0</v>
       </c>
       <c r="H1304" t="s">
-        <v>1417</v>
+        <v>1416</v>
       </c>
       <c r="I1304" t="s">
         <v>19</v>
@@ -65964,7 +65985,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -65981,19 +66002,19 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>1417</v>
+      </c>
+      <c r="F1" t="s">
         <v>1418</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>1419</v>
-      </c>
-      <c r="G1" t="s">
-        <v>1420</v>
       </c>
       <c r="H1" t="s">
         <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>1421</v>
+        <v>1420</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -66001,7 +66022,7 @@
         <v>8866</v>
       </c>
       <c r="B2" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="C2" t="s">
         <v>1163</v>
@@ -66010,7 +66031,7 @@
         <v>40</v>
       </c>
       <c r="E2" t="s">
-        <v>1422</v>
+        <v>1421</v>
       </c>
       <c r="F2">
         <v>200</v>
@@ -66019,10 +66040,10 @@
         <v>200</v>
       </c>
       <c r="H2" t="s">
+        <v>1422</v>
+      </c>
+      <c r="I2" t="s">
         <v>1423</v>
-      </c>
-      <c r="I2" t="s">
-        <v>1424</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -66030,7 +66051,7 @@
         <v>83772</v>
       </c>
       <c r="B3" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="C3" t="s">
         <v>1163</v>
@@ -66039,7 +66060,7 @@
         <v>40</v>
       </c>
       <c r="E3" t="s">
-        <v>1425</v>
+        <v>1424</v>
       </c>
       <c r="F3">
         <v>100</v>
@@ -66048,10 +66069,10 @@
         <v>100</v>
       </c>
       <c r="H3" t="s">
+        <v>1422</v>
+      </c>
+      <c r="I3" t="s">
         <v>1423</v>
-      </c>
-      <c r="I3" t="s">
-        <v>1424</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -66059,7 +66080,7 @@
         <v>83772</v>
       </c>
       <c r="B4" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="C4" t="s">
         <v>952</v>
@@ -66068,7 +66089,7 @@
         <v>40</v>
       </c>
       <c r="E4" t="s">
-        <v>1422</v>
+        <v>1421</v>
       </c>
       <c r="F4">
         <v>200</v>
@@ -66077,10 +66098,10 @@
         <v>200</v>
       </c>
       <c r="H4" t="s">
+        <v>1422</v>
+      </c>
+      <c r="I4" t="s">
         <v>1423</v>
-      </c>
-      <c r="I4" t="s">
-        <v>1424</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -66088,7 +66109,7 @@
         <v>83772</v>
       </c>
       <c r="B5" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="C5" t="s">
         <v>952</v>
@@ -66097,19 +66118,19 @@
         <v>40</v>
       </c>
       <c r="E5" t="s">
+        <v>1425</v>
+      </c>
+      <c r="F5" t="s">
         <v>1426</v>
-      </c>
-      <c r="F5" t="s">
-        <v>1427</v>
       </c>
       <c r="G5">
         <v>150</v>
       </c>
       <c r="H5" t="s">
-        <v>1428</v>
+        <v>1427</v>
       </c>
       <c r="I5" t="s">
-        <v>1424</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -66117,7 +66138,7 @@
         <v>83772</v>
       </c>
       <c r="B6" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="C6" t="s">
         <v>1163</v>
@@ -66126,7 +66147,7 @@
         <v>40</v>
       </c>
       <c r="E6" t="s">
-        <v>1429</v>
+        <v>1428</v>
       </c>
       <c r="F6">
         <v>6330</v>
@@ -66135,10 +66156,10 @@
         <v>6330</v>
       </c>
       <c r="H6" t="s">
-        <v>1423</v>
+        <v>1422</v>
       </c>
       <c r="I6" t="s">
-        <v>1430</v>
+        <v>1429</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -66146,7 +66167,7 @@
         <v>83772</v>
       </c>
       <c r="B7" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="C7" t="s">
         <v>1163</v>
@@ -66155,7 +66176,7 @@
         <v>40</v>
       </c>
       <c r="E7" t="s">
-        <v>1425</v>
+        <v>1424</v>
       </c>
       <c r="F7">
         <v>100</v>
@@ -66164,10 +66185,10 @@
         <v>100</v>
       </c>
       <c r="H7" t="s">
-        <v>1423</v>
+        <v>1422</v>
       </c>
       <c r="I7" t="s">
-        <v>1430</v>
+        <v>1429</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -66175,7 +66196,7 @@
         <v>83772</v>
       </c>
       <c r="B8" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="C8" t="s">
         <v>952</v>
@@ -66184,7 +66205,7 @@
         <v>40</v>
       </c>
       <c r="E8" t="s">
-        <v>1431</v>
+        <v>1430</v>
       </c>
       <c r="F8">
         <v>50</v>
@@ -66193,10 +66214,10 @@
         <v>50</v>
       </c>
       <c r="H8" t="s">
-        <v>1423</v>
+        <v>1422</v>
       </c>
       <c r="I8" t="s">
-        <v>1430</v>
+        <v>1429</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -66204,7 +66225,7 @@
         <v>83772</v>
       </c>
       <c r="B9" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="C9" t="s">
         <v>952</v>
@@ -66213,7 +66234,7 @@
         <v>40</v>
       </c>
       <c r="E9" t="s">
-        <v>1432</v>
+        <v>1431</v>
       </c>
       <c r="F9">
         <v>50</v>
@@ -66222,10 +66243,10 @@
         <v>50</v>
       </c>
       <c r="H9" t="s">
-        <v>1423</v>
+        <v>1422</v>
       </c>
       <c r="I9" t="s">
-        <v>1430</v>
+        <v>1429</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -66233,7 +66254,7 @@
         <v>83772</v>
       </c>
       <c r="B10" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="C10" t="s">
         <v>1163</v>
@@ -66242,7 +66263,7 @@
         <v>40</v>
       </c>
       <c r="E10" t="s">
-        <v>1425</v>
+        <v>1424</v>
       </c>
       <c r="F10">
         <v>100</v>
@@ -66251,10 +66272,10 @@
         <v>100</v>
       </c>
       <c r="H10" t="s">
-        <v>1433</v>
+        <v>1432</v>
       </c>
       <c r="I10" t="s">
-        <v>1424</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -66262,7 +66283,7 @@
         <v>8854</v>
       </c>
       <c r="B11" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="C11" t="s">
         <v>952</v>
@@ -66271,7 +66292,7 @@
         <v>339</v>
       </c>
       <c r="E11" t="s">
-        <v>1434</v>
+        <v>1433</v>
       </c>
       <c r="F11">
         <v>4000</v>
@@ -66280,10 +66301,10 @@
         <v>4000</v>
       </c>
       <c r="H11" t="s">
-        <v>1433</v>
+        <v>1432</v>
       </c>
       <c r="I11" t="s">
-        <v>1424</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -66291,7 +66312,7 @@
         <v>8854</v>
       </c>
       <c r="B12" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="C12" t="s">
         <v>952</v>
@@ -66300,7 +66321,7 @@
         <v>339</v>
       </c>
       <c r="E12" t="s">
-        <v>1434</v>
+        <v>1433</v>
       </c>
       <c r="F12">
         <v>3000</v>
@@ -66309,10 +66330,213 @@
         <v>3000</v>
       </c>
       <c r="H12" t="s">
-        <v>1433</v>
+        <v>1432</v>
       </c>
       <c r="I12" t="s">
+        <v>1423</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13">
+        <v>8839</v>
+      </c>
+      <c r="B13" t="s">
+        <v>1162</v>
+      </c>
+      <c r="C13" t="s">
+        <v>952</v>
+      </c>
+      <c r="D13" t="s">
+        <v>339</v>
+      </c>
+      <c r="E13" t="s">
+        <v>1430</v>
+      </c>
+      <c r="F13">
+        <v>50</v>
+      </c>
+      <c r="G13">
+        <v>50</v>
+      </c>
+      <c r="H13" t="s">
+        <v>1434</v>
+      </c>
+      <c r="I13" t="s">
+        <v>1423</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14">
+        <v>8839</v>
+      </c>
+      <c r="B14" t="s">
+        <v>1435</v>
+      </c>
+      <c r="C14" t="s">
+        <v>952</v>
+      </c>
+      <c r="D14" t="s">
+        <v>21</v>
+      </c>
+      <c r="E14" t="s">
+        <v>1436</v>
+      </c>
+      <c r="F14" t="s">
+        <v>1437</v>
+      </c>
+      <c r="G14">
+        <v>300</v>
+      </c>
+      <c r="H14" t="s">
+        <v>1434</v>
+      </c>
+      <c r="I14" t="s">
+        <v>1423</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15">
+        <v>8839</v>
+      </c>
+      <c r="B15" t="s">
+        <v>1435</v>
+      </c>
+      <c r="C15" t="s">
+        <v>952</v>
+      </c>
+      <c r="D15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E15" t="s">
+        <v>1421</v>
+      </c>
+      <c r="F15">
+        <v>200</v>
+      </c>
+      <c r="G15">
+        <v>200</v>
+      </c>
+      <c r="H15" t="s">
+        <v>1434</v>
+      </c>
+      <c r="I15" t="s">
+        <v>1423</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16">
+        <v>5569</v>
+      </c>
+      <c r="B16" t="s">
+        <v>1162</v>
+      </c>
+      <c r="C16" t="s">
+        <v>1163</v>
+      </c>
+      <c r="D16" t="s">
+        <v>339</v>
+      </c>
+      <c r="E16" t="s">
+        <v>1438</v>
+      </c>
+      <c r="F16">
+        <v>30</v>
+      </c>
+      <c r="G16">
+        <v>30</v>
+      </c>
+      <c r="H16" t="s">
+        <v>1439</v>
+      </c>
+      <c r="I16" t="s">
+        <v>1423</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17">
+        <v>8839</v>
+      </c>
+      <c r="B17" t="s">
+        <v>1162</v>
+      </c>
+      <c r="C17" t="s">
+        <v>952</v>
+      </c>
+      <c r="D17" t="s">
+        <v>339</v>
+      </c>
+      <c r="E17" t="s">
         <v>1424</v>
+      </c>
+      <c r="F17">
+        <v>100</v>
+      </c>
+      <c r="G17">
+        <v>100</v>
+      </c>
+      <c r="H17" t="s">
+        <v>1434</v>
+      </c>
+      <c r="I17" t="s">
+        <v>1429</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18">
+        <v>8839</v>
+      </c>
+      <c r="B18" t="s">
+        <v>1162</v>
+      </c>
+      <c r="C18" t="s">
+        <v>952</v>
+      </c>
+      <c r="D18" t="s">
+        <v>339</v>
+      </c>
+      <c r="E18" t="s">
+        <v>1424</v>
+      </c>
+      <c r="F18">
+        <v>100</v>
+      </c>
+      <c r="G18">
+        <v>100</v>
+      </c>
+      <c r="H18" t="s">
+        <v>1434</v>
+      </c>
+      <c r="I18" t="s">
+        <v>1429</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19">
+        <v>8839</v>
+      </c>
+      <c r="B19" t="s">
+        <v>1162</v>
+      </c>
+      <c r="C19" t="s">
+        <v>952</v>
+      </c>
+      <c r="D19" t="s">
+        <v>339</v>
+      </c>
+      <c r="E19" t="s">
+        <v>1440</v>
+      </c>
+      <c r="F19">
+        <v>4000</v>
+      </c>
+      <c r="G19">
+        <v>4000</v>
+      </c>
+      <c r="H19" t="s">
+        <v>1441</v>
+      </c>
+      <c r="I19" t="s">
+        <v>1429</v>
       </c>
     </row>
   </sheetData>

</xml_diff>